<commit_message>
Update Nalco PDF (2026-09-08 08:14:02 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F69"/>
+  <dimension ref="A1:F70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -466,7 +466,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -479,22 +479,22 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>361.65</v>
+        <v>365.25</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>02-09-2026</t>
+          <t>08-09-2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2026/09/Ingot-01-09-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-8-9-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
@@ -507,22 +507,22 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>360.15</v>
+        <v>361.65</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>28-08-2026</t>
+          <t>02-09-2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-08-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/09/Ingot-01-09-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
@@ -535,22 +535,22 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>356.25</v>
+        <v>360.15</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>21-08-2026</t>
+          <t>28-08-2026</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-21-08-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-08-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
@@ -563,22 +563,22 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>362.35</v>
+        <v>356.25</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>15-08-2026</t>
+          <t>21-08-2026</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-15-08-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-21-08-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
@@ -591,22 +591,22 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>375.25</v>
+        <v>362.35</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>12-08-2026</t>
+          <t>15-08-2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-12-08-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-15-08-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
@@ -619,22 +619,22 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>363.35</v>
+        <v>375.25</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>01-08-2026</t>
+          <t>12-08-2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-08-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-12-08-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
@@ -647,22 +647,22 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>354.95</v>
+        <v>363.35</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>29-07-2026</t>
+          <t>01-08-2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-08-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
@@ -675,22 +675,22 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>361.15</v>
+        <v>354.95</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>24-07-2026</t>
+          <t>29-07-2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-07-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
@@ -703,22 +703,22 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>356.35</v>
+        <v>361.15</v>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>18-07-2026</t>
+          <t>24-07-2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-07-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
@@ -731,22 +731,22 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>352.85</v>
+        <v>356.35</v>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>11-07-2026</t>
+          <t>18-07-2026</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
@@ -759,22 +759,22 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>349.05</v>
+        <v>352.85</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>08-07-2026</t>
+          <t>11-07-2026</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-08-07-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
@@ -787,22 +787,22 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>344.05</v>
+        <v>349.05</v>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>01-07-2026</t>
+          <t>08-07-2026</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-08-07-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
@@ -815,22 +815,22 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>349.05</v>
+        <v>344.05</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>29-06-2026</t>
+          <t>01-07-2026</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
@@ -847,18 +847,18 @@
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>26-06-2026</t>
+          <t>29-06-2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
@@ -871,22 +871,22 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>376.55</v>
+        <v>349.05</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>18-06-2026</t>
+          <t>26-06-2026</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
@@ -914,7 +914,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
@@ -927,22 +927,22 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>393.85</v>
+        <v>376.55</v>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>13-06-2026</t>
+          <t>18-06-2026</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
@@ -955,22 +955,22 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>402.35</v>
+        <v>393.85</v>
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>10-06-2026</t>
+          <t>13-06-2026</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-10-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
@@ -983,22 +983,22 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>416.35</v>
+        <v>402.35</v>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>05-06-2026</t>
+          <t>10-06-2026</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-10-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
@@ -1011,22 +1011,22 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>412.55</v>
+        <v>416.35</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>01-06-2026</t>
+          <t>05-06-2026</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
@@ -1039,22 +1039,22 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>411.05</v>
+        <v>412.55</v>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>27-05-2026</t>
+          <t>01-06-2026</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
@@ -1067,22 +1067,22 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>404.95</v>
+        <v>411.05</v>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>20-05-2026</t>
+          <t>27-05-2026</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
@@ -1095,22 +1095,22 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>408.85</v>
+        <v>404.95</v>
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>14-05-2026</t>
+          <t>20-05-2026</t>
         </is>
       </c>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
@@ -1123,22 +1123,22 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>390.05</v>
+        <v>408.85</v>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>01-05-2026</t>
+          <t>14-05-2026</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
@@ -1151,22 +1151,22 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>392.55</v>
+        <v>390.05</v>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>24-04-2026</t>
+          <t>01-05-2026</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
@@ -1179,22 +1179,22 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>383.65</v>
+        <v>392.55</v>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>16-04-2026</t>
+          <t>24-04-2026</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
@@ -1207,22 +1207,22 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>373.55</v>
+        <v>383.65</v>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>03-04-2026</t>
+          <t>16-04-2026</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
@@ -1235,22 +1235,22 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>357.05</v>
+        <v>373.55</v>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>28-03-2026</t>
+          <t>03-04-2026</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
@@ -1263,22 +1263,22 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>350.45</v>
+        <v>357.05</v>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>24-03-2026</t>
+          <t>28-03-2026</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
@@ -1291,22 +1291,22 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>360.05</v>
+        <v>350.45</v>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>19-03-2026</t>
+          <t>24-03-2026</t>
         </is>
       </c>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
@@ -1319,22 +1319,22 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>372.05</v>
+        <v>360.05</v>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>14-03-2026</t>
+          <t>19-03-2026</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
@@ -1347,22 +1347,22 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>358.75</v>
+        <v>372.05</v>
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>11-03-2026</t>
+          <t>14-03-2026</t>
         </is>
       </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
@@ -1375,22 +1375,22 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>347.25</v>
+        <v>358.75</v>
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>06-03-2026</t>
+          <t>11-03-2026</t>
         </is>
       </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
@@ -1403,22 +1403,22 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>339.45</v>
+        <v>347.25</v>
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>06-03-2026</t>
         </is>
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
@@ -1431,22 +1431,22 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>330.95</v>
+        <v>339.45</v>
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
@@ -1459,22 +1459,22 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>323.05</v>
+        <v>330.95</v>
       </c>
       <c r="E37" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="F37" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
@@ -1487,22 +1487,22 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>316.15</v>
+        <v>323.05</v>
       </c>
       <c r="E38" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="F38" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
@@ -1515,22 +1515,22 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>323.75</v>
+        <v>316.15</v>
       </c>
       <c r="E39" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="F39" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B40" s="1" t="inlineStr">
         <is>
@@ -1543,22 +1543,22 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>318.05</v>
+        <v>323.75</v>
       </c>
       <c r="E40" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="F40" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B41" s="1" t="inlineStr">
         <is>
@@ -1571,22 +1571,22 @@
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>320.45</v>
+        <v>318.05</v>
       </c>
       <c r="E41" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="F41" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B42" s="1" t="inlineStr">
         <is>
@@ -1599,22 +1599,22 @@
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E42" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F42" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B43" s="1" t="inlineStr">
         <is>
@@ -1627,22 +1627,22 @@
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E43" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F43" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="B44" s="1" t="inlineStr">
         <is>
@@ -1655,22 +1655,22 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E44" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F44" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B45" s="1" t="inlineStr">
         <is>
@@ -1683,22 +1683,22 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E45" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F45" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B46" s="1" t="inlineStr">
         <is>
@@ -1711,22 +1711,22 @@
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>307.25</v>
+        <v>320.05</v>
       </c>
       <c r="E46" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="F46" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B47" s="1" t="inlineStr">
         <is>
@@ -1739,22 +1739,22 @@
         </is>
       </c>
       <c r="D47" s="2" t="n">
-        <v>301.65</v>
+        <v>307.25</v>
       </c>
       <c r="E47" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F47" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B48" s="1" t="inlineStr">
         <is>
@@ -1767,22 +1767,22 @@
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>296.05</v>
+        <v>301.65</v>
       </c>
       <c r="E48" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="F48" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B49" s="1" t="inlineStr">
         <is>
@@ -1795,22 +1795,22 @@
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>290.95</v>
+        <v>296.05</v>
       </c>
       <c r="E49" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="F49" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B50" s="1" t="inlineStr">
         <is>
@@ -1823,22 +1823,22 @@
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>283.55</v>
+        <v>290.95</v>
       </c>
       <c r="E50" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="F50" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B51" s="1" t="inlineStr">
         <is>
@@ -1851,22 +1851,22 @@
         </is>
       </c>
       <c r="D51" s="2" t="n">
-        <v>281.95</v>
+        <v>283.55</v>
       </c>
       <c r="E51" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="F51" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B52" s="1" t="inlineStr">
         <is>
@@ -1879,22 +1879,22 @@
         </is>
       </c>
       <c r="D52" s="2" t="n">
-        <v>292.65</v>
+        <v>281.95</v>
       </c>
       <c r="E52" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="F52" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B53" s="1" t="inlineStr">
         <is>
@@ -1907,22 +1907,22 @@
         </is>
       </c>
       <c r="D53" s="2" t="n">
-        <v>296.05</v>
+        <v>292.65</v>
       </c>
       <c r="E53" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="F53" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B54" s="1" t="inlineStr">
         <is>
@@ -1935,22 +1935,22 @@
         </is>
       </c>
       <c r="D54" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E54" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F54" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B55" s="1" t="inlineStr">
         <is>
@@ -1963,22 +1963,22 @@
         </is>
       </c>
       <c r="D55" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E55" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F55" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B56" s="1" t="inlineStr">
         <is>
@@ -1991,22 +1991,22 @@
         </is>
       </c>
       <c r="D56" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E56" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F56" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B57" s="1" t="inlineStr">
         <is>
@@ -2019,22 +2019,22 @@
         </is>
       </c>
       <c r="D57" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E57" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F57" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B58" s="1" t="inlineStr">
         <is>
@@ -2047,22 +2047,22 @@
         </is>
       </c>
       <c r="D58" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E58" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F58" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B59" s="1" t="inlineStr">
         <is>
@@ -2075,22 +2075,22 @@
         </is>
       </c>
       <c r="D59" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E59" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F59" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B60" s="1" t="inlineStr">
         <is>
@@ -2103,22 +2103,22 @@
         </is>
       </c>
       <c r="D60" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E60" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F60" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B61" s="1" t="inlineStr">
         <is>
@@ -2131,22 +2131,22 @@
         </is>
       </c>
       <c r="D61" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E61" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F61" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B62" s="1" t="inlineStr">
         <is>
@@ -2159,22 +2159,22 @@
         </is>
       </c>
       <c r="D62" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E62" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F62" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="1" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B63" s="1" t="inlineStr">
         <is>
@@ -2187,22 +2187,22 @@
         </is>
       </c>
       <c r="D63" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E63" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F63" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="1" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B64" s="1" t="inlineStr">
         <is>
@@ -2215,22 +2215,22 @@
         </is>
       </c>
       <c r="D64" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E64" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F64" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B65" s="1" t="inlineStr">
         <is>
@@ -2243,22 +2243,22 @@
         </is>
       </c>
       <c r="D65" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E65" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F65" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B66" s="1" t="inlineStr">
         <is>
@@ -2271,22 +2271,22 @@
         </is>
       </c>
       <c r="D66" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E66" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F66" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="1" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B67" s="1" t="inlineStr">
         <is>
@@ -2299,22 +2299,22 @@
         </is>
       </c>
       <c r="D67" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E67" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F67" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B68" s="1" t="inlineStr">
         <is>
@@ -2327,42 +2327,70 @@
         </is>
       </c>
       <c r="D68" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E68" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F68" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B69" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C69" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="n">
+        <v>269.45</v>
+      </c>
+      <c r="E69" s="1" t="inlineStr">
+        <is>
+          <t>15-08-2025</t>
+        </is>
+      </c>
+      <c r="F69" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B69" s="1" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C69" s="1" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D69" s="2" t="n">
+      <c r="B70" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C70" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="n">
         <v>268.25</v>
       </c>
-      <c r="E69" s="1" t="inlineStr">
+      <c r="E70" s="1" t="inlineStr">
         <is>
           <t>07-08-2025</t>
         </is>
       </c>
-      <c r="F69" s="1" t="inlineStr">
+      <c r="F70" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
@@ -2438,6 +2466,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F67" r:id="rId66"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F68" r:id="rId67"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F69" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F70" r:id="rId69"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-09-11 11:02:54 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F70"/>
+  <dimension ref="A1:F71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -466,7 +466,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -479,22 +479,22 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>365.25</v>
+        <v>371.55</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>08-09-2026</t>
+          <t>11-09-2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-8-9-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-09-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
@@ -507,22 +507,22 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>361.65</v>
+        <v>365.25</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>02-09-2026</t>
+          <t>08-09-2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2026/09/Ingot-01-09-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-8-9-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
@@ -535,22 +535,22 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>360.15</v>
+        <v>361.65</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>28-08-2026</t>
+          <t>02-09-2026</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-08-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/09/Ingot-01-09-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
@@ -563,22 +563,22 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>356.25</v>
+        <v>360.15</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>21-08-2026</t>
+          <t>28-08-2026</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-21-08-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-08-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
@@ -591,22 +591,22 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>362.35</v>
+        <v>356.25</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>15-08-2026</t>
+          <t>21-08-2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-15-08-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-21-08-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
@@ -619,22 +619,22 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>375.25</v>
+        <v>362.35</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>12-08-2026</t>
+          <t>15-08-2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-12-08-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-15-08-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
@@ -647,22 +647,22 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>363.35</v>
+        <v>375.25</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>01-08-2026</t>
+          <t>12-08-2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-08-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-12-08-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
@@ -675,22 +675,22 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>354.95</v>
+        <v>363.35</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>29-07-2026</t>
+          <t>01-08-2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-08-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
@@ -703,22 +703,22 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>361.15</v>
+        <v>354.95</v>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>24-07-2026</t>
+          <t>29-07-2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-07-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
@@ -731,22 +731,22 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>356.35</v>
+        <v>361.15</v>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>18-07-2026</t>
+          <t>24-07-2026</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-07-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
@@ -759,22 +759,22 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>352.85</v>
+        <v>356.35</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>11-07-2026</t>
+          <t>18-07-2026</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
@@ -787,22 +787,22 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>349.05</v>
+        <v>352.85</v>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>08-07-2026</t>
+          <t>11-07-2026</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-08-07-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
@@ -815,22 +815,22 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>344.05</v>
+        <v>349.05</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>01-07-2026</t>
+          <t>08-07-2026</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-08-07-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
@@ -843,22 +843,22 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>349.05</v>
+        <v>344.05</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>29-06-2026</t>
+          <t>01-07-2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
@@ -875,18 +875,18 @@
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>26-06-2026</t>
+          <t>29-06-2026</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
@@ -899,22 +899,22 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>376.55</v>
+        <v>349.05</v>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>18-06-2026</t>
+          <t>26-06-2026</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
@@ -942,7 +942,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
@@ -955,22 +955,22 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>393.85</v>
+        <v>376.55</v>
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>13-06-2026</t>
+          <t>18-06-2026</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
@@ -983,22 +983,22 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>402.35</v>
+        <v>393.85</v>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>10-06-2026</t>
+          <t>13-06-2026</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-10-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
@@ -1011,22 +1011,22 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>416.35</v>
+        <v>402.35</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>05-06-2026</t>
+          <t>10-06-2026</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-10-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
@@ -1039,22 +1039,22 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>412.55</v>
+        <v>416.35</v>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>01-06-2026</t>
+          <t>05-06-2026</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
@@ -1067,22 +1067,22 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>411.05</v>
+        <v>412.55</v>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>27-05-2026</t>
+          <t>01-06-2026</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
@@ -1095,22 +1095,22 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>404.95</v>
+        <v>411.05</v>
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>20-05-2026</t>
+          <t>27-05-2026</t>
         </is>
       </c>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
@@ -1123,22 +1123,22 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>408.85</v>
+        <v>404.95</v>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>14-05-2026</t>
+          <t>20-05-2026</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
@@ -1151,22 +1151,22 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>390.05</v>
+        <v>408.85</v>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>01-05-2026</t>
+          <t>14-05-2026</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
@@ -1179,22 +1179,22 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>392.55</v>
+        <v>390.05</v>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>24-04-2026</t>
+          <t>01-05-2026</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
@@ -1207,22 +1207,22 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>383.65</v>
+        <v>392.55</v>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>16-04-2026</t>
+          <t>24-04-2026</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
@@ -1235,22 +1235,22 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>373.55</v>
+        <v>383.65</v>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>03-04-2026</t>
+          <t>16-04-2026</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
@@ -1263,22 +1263,22 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>357.05</v>
+        <v>373.55</v>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>28-03-2026</t>
+          <t>03-04-2026</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
@@ -1291,22 +1291,22 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>350.45</v>
+        <v>357.05</v>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>24-03-2026</t>
+          <t>28-03-2026</t>
         </is>
       </c>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
@@ -1319,22 +1319,22 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>360.05</v>
+        <v>350.45</v>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>19-03-2026</t>
+          <t>24-03-2026</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
@@ -1347,22 +1347,22 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>372.05</v>
+        <v>360.05</v>
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>14-03-2026</t>
+          <t>19-03-2026</t>
         </is>
       </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
@@ -1375,22 +1375,22 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>358.75</v>
+        <v>372.05</v>
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>11-03-2026</t>
+          <t>14-03-2026</t>
         </is>
       </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
@@ -1403,22 +1403,22 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>347.25</v>
+        <v>358.75</v>
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>06-03-2026</t>
+          <t>11-03-2026</t>
         </is>
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
@@ -1431,22 +1431,22 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>339.45</v>
+        <v>347.25</v>
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>06-03-2026</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
@@ -1459,22 +1459,22 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>330.95</v>
+        <v>339.45</v>
       </c>
       <c r="E37" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F37" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
@@ -1487,22 +1487,22 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>323.05</v>
+        <v>330.95</v>
       </c>
       <c r="E38" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="F38" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
@@ -1515,22 +1515,22 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>316.15</v>
+        <v>323.05</v>
       </c>
       <c r="E39" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="F39" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B40" s="1" t="inlineStr">
         <is>
@@ -1543,22 +1543,22 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>323.75</v>
+        <v>316.15</v>
       </c>
       <c r="E40" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="F40" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B41" s="1" t="inlineStr">
         <is>
@@ -1571,22 +1571,22 @@
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>318.05</v>
+        <v>323.75</v>
       </c>
       <c r="E41" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="F41" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B42" s="1" t="inlineStr">
         <is>
@@ -1599,22 +1599,22 @@
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>320.45</v>
+        <v>318.05</v>
       </c>
       <c r="E42" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="F42" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B43" s="1" t="inlineStr">
         <is>
@@ -1627,22 +1627,22 @@
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E43" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F43" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B44" s="1" t="inlineStr">
         <is>
@@ -1655,22 +1655,22 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E44" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F44" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="B45" s="1" t="inlineStr">
         <is>
@@ -1683,22 +1683,22 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E45" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F45" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B46" s="1" t="inlineStr">
         <is>
@@ -1711,22 +1711,22 @@
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E46" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F46" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B47" s="1" t="inlineStr">
         <is>
@@ -1739,22 +1739,22 @@
         </is>
       </c>
       <c r="D47" s="2" t="n">
-        <v>307.25</v>
+        <v>320.05</v>
       </c>
       <c r="E47" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="F47" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B48" s="1" t="inlineStr">
         <is>
@@ -1767,22 +1767,22 @@
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>301.65</v>
+        <v>307.25</v>
       </c>
       <c r="E48" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F48" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B49" s="1" t="inlineStr">
         <is>
@@ -1795,22 +1795,22 @@
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>296.05</v>
+        <v>301.65</v>
       </c>
       <c r="E49" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="F49" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B50" s="1" t="inlineStr">
         <is>
@@ -1823,22 +1823,22 @@
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>290.95</v>
+        <v>296.05</v>
       </c>
       <c r="E50" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="F50" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B51" s="1" t="inlineStr">
         <is>
@@ -1851,22 +1851,22 @@
         </is>
       </c>
       <c r="D51" s="2" t="n">
-        <v>283.55</v>
+        <v>290.95</v>
       </c>
       <c r="E51" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="F51" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B52" s="1" t="inlineStr">
         <is>
@@ -1879,22 +1879,22 @@
         </is>
       </c>
       <c r="D52" s="2" t="n">
-        <v>281.95</v>
+        <v>283.55</v>
       </c>
       <c r="E52" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="F52" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B53" s="1" t="inlineStr">
         <is>
@@ -1907,22 +1907,22 @@
         </is>
       </c>
       <c r="D53" s="2" t="n">
-        <v>292.65</v>
+        <v>281.95</v>
       </c>
       <c r="E53" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="F53" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B54" s="1" t="inlineStr">
         <is>
@@ -1935,22 +1935,22 @@
         </is>
       </c>
       <c r="D54" s="2" t="n">
-        <v>296.05</v>
+        <v>292.65</v>
       </c>
       <c r="E54" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="F54" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B55" s="1" t="inlineStr">
         <is>
@@ -1963,22 +1963,22 @@
         </is>
       </c>
       <c r="D55" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E55" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F55" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B56" s="1" t="inlineStr">
         <is>
@@ -1991,22 +1991,22 @@
         </is>
       </c>
       <c r="D56" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E56" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F56" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B57" s="1" t="inlineStr">
         <is>
@@ -2019,22 +2019,22 @@
         </is>
       </c>
       <c r="D57" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E57" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F57" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B58" s="1" t="inlineStr">
         <is>
@@ -2047,22 +2047,22 @@
         </is>
       </c>
       <c r="D58" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E58" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F58" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B59" s="1" t="inlineStr">
         <is>
@@ -2075,22 +2075,22 @@
         </is>
       </c>
       <c r="D59" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E59" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F59" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B60" s="1" t="inlineStr">
         <is>
@@ -2103,22 +2103,22 @@
         </is>
       </c>
       <c r="D60" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E60" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F60" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B61" s="1" t="inlineStr">
         <is>
@@ -2131,22 +2131,22 @@
         </is>
       </c>
       <c r="D61" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E61" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F61" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B62" s="1" t="inlineStr">
         <is>
@@ -2159,22 +2159,22 @@
         </is>
       </c>
       <c r="D62" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E62" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F62" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="1" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B63" s="1" t="inlineStr">
         <is>
@@ -2187,22 +2187,22 @@
         </is>
       </c>
       <c r="D63" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E63" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F63" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="1" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B64" s="1" t="inlineStr">
         <is>
@@ -2215,22 +2215,22 @@
         </is>
       </c>
       <c r="D64" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E64" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F64" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="1" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B65" s="1" t="inlineStr">
         <is>
@@ -2243,22 +2243,22 @@
         </is>
       </c>
       <c r="D65" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E65" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F65" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B66" s="1" t="inlineStr">
         <is>
@@ -2271,22 +2271,22 @@
         </is>
       </c>
       <c r="D66" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E66" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F66" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B67" s="1" t="inlineStr">
         <is>
@@ -2299,22 +2299,22 @@
         </is>
       </c>
       <c r="D67" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E67" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F67" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="1" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B68" s="1" t="inlineStr">
         <is>
@@ -2327,22 +2327,22 @@
         </is>
       </c>
       <c r="D68" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E68" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F68" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B69" s="1" t="inlineStr">
         <is>
@@ -2355,42 +2355,70 @@
         </is>
       </c>
       <c r="D69" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E69" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F69" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B70" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C70" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="n">
+        <v>269.45</v>
+      </c>
+      <c r="E70" s="1" t="inlineStr">
+        <is>
+          <t>15-08-2025</t>
+        </is>
+      </c>
+      <c r="F70" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B70" s="1" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C70" s="1" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D70" s="2" t="n">
+      <c r="B71" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C71" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="n">
         <v>268.25</v>
       </c>
-      <c r="E70" s="1" t="inlineStr">
+      <c r="E71" s="1" t="inlineStr">
         <is>
           <t>07-08-2025</t>
         </is>
       </c>
-      <c r="F70" s="1" t="inlineStr">
+      <c r="F71" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
@@ -2467,6 +2495,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F68" r:id="rId67"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F69" r:id="rId68"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F70" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F71" r:id="rId70"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-09-16 08:44:37 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F71"/>
+  <dimension ref="A1:F72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -466,7 +466,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -479,22 +479,22 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>371.55</v>
+        <v>365.55</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>11-09-2026</t>
+          <t>16-09-2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-09-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-09-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
@@ -507,22 +507,22 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>365.25</v>
+        <v>371.55</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>08-09-2026</t>
+          <t>11-09-2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-8-9-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-09-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
@@ -535,22 +535,22 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>361.65</v>
+        <v>365.25</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>02-09-2026</t>
+          <t>08-09-2026</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2026/09/Ingot-01-09-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-8-9-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
@@ -563,22 +563,22 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>360.15</v>
+        <v>361.65</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>28-08-2026</t>
+          <t>02-09-2026</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-08-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/09/Ingot-01-09-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
@@ -591,22 +591,22 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>356.25</v>
+        <v>360.15</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>21-08-2026</t>
+          <t>28-08-2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-21-08-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-08-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
@@ -619,22 +619,22 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>362.35</v>
+        <v>356.25</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>15-08-2026</t>
+          <t>21-08-2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-15-08-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-21-08-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
@@ -647,22 +647,22 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>375.25</v>
+        <v>362.35</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>12-08-2026</t>
+          <t>15-08-2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-12-08-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-15-08-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
@@ -675,22 +675,22 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>363.35</v>
+        <v>375.25</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>01-08-2026</t>
+          <t>12-08-2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-08-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-12-08-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
@@ -703,22 +703,22 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>354.95</v>
+        <v>363.35</v>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>29-07-2026</t>
+          <t>01-08-2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-08-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
@@ -731,22 +731,22 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>361.15</v>
+        <v>354.95</v>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>24-07-2026</t>
+          <t>29-07-2026</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-07-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
@@ -759,22 +759,22 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>356.35</v>
+        <v>361.15</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>18-07-2026</t>
+          <t>24-07-2026</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-07-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
@@ -787,22 +787,22 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>352.85</v>
+        <v>356.35</v>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>11-07-2026</t>
+          <t>18-07-2026</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
@@ -815,22 +815,22 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>349.05</v>
+        <v>352.85</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>08-07-2026</t>
+          <t>11-07-2026</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-08-07-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
@@ -843,22 +843,22 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>344.05</v>
+        <v>349.05</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>01-07-2026</t>
+          <t>08-07-2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-08-07-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
@@ -871,22 +871,22 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>349.05</v>
+        <v>344.05</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>29-06-2026</t>
+          <t>01-07-2026</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
@@ -903,18 +903,18 @@
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>26-06-2026</t>
+          <t>29-06-2026</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
@@ -927,22 +927,22 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>376.55</v>
+        <v>349.05</v>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>18-06-2026</t>
+          <t>26-06-2026</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
@@ -970,7 +970,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
@@ -983,22 +983,22 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>393.85</v>
+        <v>376.55</v>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>13-06-2026</t>
+          <t>18-06-2026</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
@@ -1011,22 +1011,22 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>402.35</v>
+        <v>393.85</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>10-06-2026</t>
+          <t>13-06-2026</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-10-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
@@ -1039,22 +1039,22 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>416.35</v>
+        <v>402.35</v>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>05-06-2026</t>
+          <t>10-06-2026</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-10-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
@@ -1067,22 +1067,22 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>412.55</v>
+        <v>416.35</v>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>01-06-2026</t>
+          <t>05-06-2026</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
@@ -1095,22 +1095,22 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>411.05</v>
+        <v>412.55</v>
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>27-05-2026</t>
+          <t>01-06-2026</t>
         </is>
       </c>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
@@ -1123,22 +1123,22 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>404.95</v>
+        <v>411.05</v>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>20-05-2026</t>
+          <t>27-05-2026</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
@@ -1151,22 +1151,22 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>408.85</v>
+        <v>404.95</v>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>14-05-2026</t>
+          <t>20-05-2026</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
@@ -1179,22 +1179,22 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>390.05</v>
+        <v>408.85</v>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>01-05-2026</t>
+          <t>14-05-2026</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
@@ -1207,22 +1207,22 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>392.55</v>
+        <v>390.05</v>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>24-04-2026</t>
+          <t>01-05-2026</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
@@ -1235,22 +1235,22 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>383.65</v>
+        <v>392.55</v>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>16-04-2026</t>
+          <t>24-04-2026</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
@@ -1263,22 +1263,22 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>373.55</v>
+        <v>383.65</v>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>03-04-2026</t>
+          <t>16-04-2026</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
@@ -1291,22 +1291,22 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>357.05</v>
+        <v>373.55</v>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>28-03-2026</t>
+          <t>03-04-2026</t>
         </is>
       </c>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
@@ -1319,22 +1319,22 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>350.45</v>
+        <v>357.05</v>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>24-03-2026</t>
+          <t>28-03-2026</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
@@ -1347,22 +1347,22 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>360.05</v>
+        <v>350.45</v>
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>19-03-2026</t>
+          <t>24-03-2026</t>
         </is>
       </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
@@ -1375,22 +1375,22 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>372.05</v>
+        <v>360.05</v>
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>14-03-2026</t>
+          <t>19-03-2026</t>
         </is>
       </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
@@ -1403,22 +1403,22 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>358.75</v>
+        <v>372.05</v>
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>11-03-2026</t>
+          <t>14-03-2026</t>
         </is>
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
@@ -1431,22 +1431,22 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>347.25</v>
+        <v>358.75</v>
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>06-03-2026</t>
+          <t>11-03-2026</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
@@ -1459,22 +1459,22 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>339.45</v>
+        <v>347.25</v>
       </c>
       <c r="E37" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>06-03-2026</t>
         </is>
       </c>
       <c r="F37" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
@@ -1487,22 +1487,22 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>330.95</v>
+        <v>339.45</v>
       </c>
       <c r="E38" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F38" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
@@ -1515,22 +1515,22 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>323.05</v>
+        <v>330.95</v>
       </c>
       <c r="E39" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="F39" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B40" s="1" t="inlineStr">
         <is>
@@ -1543,22 +1543,22 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>316.15</v>
+        <v>323.05</v>
       </c>
       <c r="E40" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="F40" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B41" s="1" t="inlineStr">
         <is>
@@ -1571,22 +1571,22 @@
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>323.75</v>
+        <v>316.15</v>
       </c>
       <c r="E41" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="F41" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B42" s="1" t="inlineStr">
         <is>
@@ -1599,22 +1599,22 @@
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>318.05</v>
+        <v>323.75</v>
       </c>
       <c r="E42" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="F42" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B43" s="1" t="inlineStr">
         <is>
@@ -1627,22 +1627,22 @@
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>320.45</v>
+        <v>318.05</v>
       </c>
       <c r="E43" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="F43" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B44" s="1" t="inlineStr">
         <is>
@@ -1655,22 +1655,22 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E44" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F44" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B45" s="1" t="inlineStr">
         <is>
@@ -1683,22 +1683,22 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E45" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F45" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="B46" s="1" t="inlineStr">
         <is>
@@ -1711,22 +1711,22 @@
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E46" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F46" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B47" s="1" t="inlineStr">
         <is>
@@ -1739,22 +1739,22 @@
         </is>
       </c>
       <c r="D47" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E47" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F47" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B48" s="1" t="inlineStr">
         <is>
@@ -1767,22 +1767,22 @@
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>307.25</v>
+        <v>320.05</v>
       </c>
       <c r="E48" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="F48" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B49" s="1" t="inlineStr">
         <is>
@@ -1795,22 +1795,22 @@
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>301.65</v>
+        <v>307.25</v>
       </c>
       <c r="E49" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F49" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B50" s="1" t="inlineStr">
         <is>
@@ -1823,22 +1823,22 @@
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>296.05</v>
+        <v>301.65</v>
       </c>
       <c r="E50" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="F50" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B51" s="1" t="inlineStr">
         <is>
@@ -1851,22 +1851,22 @@
         </is>
       </c>
       <c r="D51" s="2" t="n">
-        <v>290.95</v>
+        <v>296.05</v>
       </c>
       <c r="E51" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="F51" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B52" s="1" t="inlineStr">
         <is>
@@ -1879,22 +1879,22 @@
         </is>
       </c>
       <c r="D52" s="2" t="n">
-        <v>283.55</v>
+        <v>290.95</v>
       </c>
       <c r="E52" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="F52" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B53" s="1" t="inlineStr">
         <is>
@@ -1907,22 +1907,22 @@
         </is>
       </c>
       <c r="D53" s="2" t="n">
-        <v>281.95</v>
+        <v>283.55</v>
       </c>
       <c r="E53" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="F53" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B54" s="1" t="inlineStr">
         <is>
@@ -1935,22 +1935,22 @@
         </is>
       </c>
       <c r="D54" s="2" t="n">
-        <v>292.65</v>
+        <v>281.95</v>
       </c>
       <c r="E54" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="F54" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B55" s="1" t="inlineStr">
         <is>
@@ -1963,22 +1963,22 @@
         </is>
       </c>
       <c r="D55" s="2" t="n">
-        <v>296.05</v>
+        <v>292.65</v>
       </c>
       <c r="E55" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="F55" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B56" s="1" t="inlineStr">
         <is>
@@ -1991,22 +1991,22 @@
         </is>
       </c>
       <c r="D56" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E56" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F56" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B57" s="1" t="inlineStr">
         <is>
@@ -2019,22 +2019,22 @@
         </is>
       </c>
       <c r="D57" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E57" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F57" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B58" s="1" t="inlineStr">
         <is>
@@ -2047,22 +2047,22 @@
         </is>
       </c>
       <c r="D58" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E58" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F58" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B59" s="1" t="inlineStr">
         <is>
@@ -2075,22 +2075,22 @@
         </is>
       </c>
       <c r="D59" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E59" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F59" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B60" s="1" t="inlineStr">
         <is>
@@ -2103,22 +2103,22 @@
         </is>
       </c>
       <c r="D60" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E60" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F60" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B61" s="1" t="inlineStr">
         <is>
@@ -2131,22 +2131,22 @@
         </is>
       </c>
       <c r="D61" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E61" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F61" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B62" s="1" t="inlineStr">
         <is>
@@ -2159,22 +2159,22 @@
         </is>
       </c>
       <c r="D62" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E62" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F62" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="1" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B63" s="1" t="inlineStr">
         <is>
@@ -2187,22 +2187,22 @@
         </is>
       </c>
       <c r="D63" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E63" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F63" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="1" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B64" s="1" t="inlineStr">
         <is>
@@ -2215,22 +2215,22 @@
         </is>
       </c>
       <c r="D64" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E64" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F64" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="1" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B65" s="1" t="inlineStr">
         <is>
@@ -2243,22 +2243,22 @@
         </is>
       </c>
       <c r="D65" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E65" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F65" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="1" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B66" s="1" t="inlineStr">
         <is>
@@ -2271,22 +2271,22 @@
         </is>
       </c>
       <c r="D66" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E66" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F66" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B67" s="1" t="inlineStr">
         <is>
@@ -2299,22 +2299,22 @@
         </is>
       </c>
       <c r="D67" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E67" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F67" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B68" s="1" t="inlineStr">
         <is>
@@ -2327,22 +2327,22 @@
         </is>
       </c>
       <c r="D68" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E68" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F68" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="1" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B69" s="1" t="inlineStr">
         <is>
@@ -2355,22 +2355,22 @@
         </is>
       </c>
       <c r="D69" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E69" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F69" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B70" s="1" t="inlineStr">
         <is>
@@ -2383,42 +2383,70 @@
         </is>
       </c>
       <c r="D70" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E70" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F70" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B71" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C71" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="n">
+        <v>269.45</v>
+      </c>
+      <c r="E71" s="1" t="inlineStr">
+        <is>
+          <t>15-08-2025</t>
+        </is>
+      </c>
+      <c r="F71" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B71" s="1" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C71" s="1" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D71" s="2" t="n">
+      <c r="B72" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C72" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="n">
         <v>268.25</v>
       </c>
-      <c r="E71" s="1" t="inlineStr">
+      <c r="E72" s="1" t="inlineStr">
         <is>
           <t>07-08-2025</t>
         </is>
       </c>
-      <c r="F71" s="1" t="inlineStr">
+      <c r="F72" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
@@ -2496,6 +2524,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F69" r:id="rId68"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F70" r:id="rId69"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F71" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F72" r:id="rId71"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-09-19 08:11:26 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F72"/>
+  <dimension ref="A1:F73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -466,7 +466,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -479,22 +479,22 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>365.55</v>
+        <v>367.65</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>16-09-2026</t>
+          <t>19-09-2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-09-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-09-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
@@ -507,22 +507,22 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>371.55</v>
+        <v>365.55</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>11-09-2026</t>
+          <t>16-09-2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-09-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-09-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
@@ -535,22 +535,22 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>365.25</v>
+        <v>371.55</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>08-09-2026</t>
+          <t>11-09-2026</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-8-9-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-09-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
@@ -563,22 +563,22 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>361.65</v>
+        <v>365.25</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>02-09-2026</t>
+          <t>08-09-2026</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2026/09/Ingot-01-09-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-8-9-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
@@ -591,22 +591,22 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>360.15</v>
+        <v>361.65</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>28-08-2026</t>
+          <t>02-09-2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-08-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/09/Ingot-01-09-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
@@ -619,22 +619,22 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>356.25</v>
+        <v>360.15</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>21-08-2026</t>
+          <t>28-08-2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-21-08-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-08-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
@@ -647,22 +647,22 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>362.35</v>
+        <v>356.25</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>15-08-2026</t>
+          <t>21-08-2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-15-08-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-21-08-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
@@ -675,22 +675,22 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>375.25</v>
+        <v>362.35</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>12-08-2026</t>
+          <t>15-08-2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-12-08-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-15-08-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
@@ -703,22 +703,22 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>363.35</v>
+        <v>375.25</v>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>01-08-2026</t>
+          <t>12-08-2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-08-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-12-08-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
@@ -731,22 +731,22 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>354.95</v>
+        <v>363.35</v>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>29-07-2026</t>
+          <t>01-08-2026</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-08-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
@@ -759,22 +759,22 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>361.15</v>
+        <v>354.95</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>24-07-2026</t>
+          <t>29-07-2026</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-07-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
@@ -787,22 +787,22 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>356.35</v>
+        <v>361.15</v>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>18-07-2026</t>
+          <t>24-07-2026</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-07-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
@@ -815,22 +815,22 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>352.85</v>
+        <v>356.35</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>11-07-2026</t>
+          <t>18-07-2026</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
@@ -843,22 +843,22 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>349.05</v>
+        <v>352.85</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>08-07-2026</t>
+          <t>11-07-2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-08-07-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
@@ -871,22 +871,22 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>344.05</v>
+        <v>349.05</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>01-07-2026</t>
+          <t>08-07-2026</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-08-07-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
@@ -899,22 +899,22 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>349.05</v>
+        <v>344.05</v>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>29-06-2026</t>
+          <t>01-07-2026</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
@@ -931,18 +931,18 @@
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>26-06-2026</t>
+          <t>29-06-2026</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
@@ -955,22 +955,22 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>376.55</v>
+        <v>349.05</v>
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>18-06-2026</t>
+          <t>26-06-2026</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
@@ -998,7 +998,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
@@ -1011,22 +1011,22 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>393.85</v>
+        <v>376.55</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>13-06-2026</t>
+          <t>18-06-2026</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
@@ -1039,22 +1039,22 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>402.35</v>
+        <v>393.85</v>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>10-06-2026</t>
+          <t>13-06-2026</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-10-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
@@ -1067,22 +1067,22 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>416.35</v>
+        <v>402.35</v>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>05-06-2026</t>
+          <t>10-06-2026</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-10-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
@@ -1095,22 +1095,22 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>412.55</v>
+        <v>416.35</v>
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>01-06-2026</t>
+          <t>05-06-2026</t>
         </is>
       </c>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
@@ -1123,22 +1123,22 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>411.05</v>
+        <v>412.55</v>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>27-05-2026</t>
+          <t>01-06-2026</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
@@ -1151,22 +1151,22 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>404.95</v>
+        <v>411.05</v>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>20-05-2026</t>
+          <t>27-05-2026</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
@@ -1179,22 +1179,22 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>408.85</v>
+        <v>404.95</v>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>14-05-2026</t>
+          <t>20-05-2026</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
@@ -1207,22 +1207,22 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>390.05</v>
+        <v>408.85</v>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>01-05-2026</t>
+          <t>14-05-2026</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
@@ -1235,22 +1235,22 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>392.55</v>
+        <v>390.05</v>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>24-04-2026</t>
+          <t>01-05-2026</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
@@ -1263,22 +1263,22 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>383.65</v>
+        <v>392.55</v>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>16-04-2026</t>
+          <t>24-04-2026</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
@@ -1291,22 +1291,22 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>373.55</v>
+        <v>383.65</v>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>03-04-2026</t>
+          <t>16-04-2026</t>
         </is>
       </c>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
@@ -1319,22 +1319,22 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>357.05</v>
+        <v>373.55</v>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>28-03-2026</t>
+          <t>03-04-2026</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
@@ -1347,22 +1347,22 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>350.45</v>
+        <v>357.05</v>
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>24-03-2026</t>
+          <t>28-03-2026</t>
         </is>
       </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
@@ -1375,22 +1375,22 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>360.05</v>
+        <v>350.45</v>
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>19-03-2026</t>
+          <t>24-03-2026</t>
         </is>
       </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
@@ -1403,22 +1403,22 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>372.05</v>
+        <v>360.05</v>
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>14-03-2026</t>
+          <t>19-03-2026</t>
         </is>
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
@@ -1431,22 +1431,22 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>358.75</v>
+        <v>372.05</v>
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>11-03-2026</t>
+          <t>14-03-2026</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
@@ -1459,22 +1459,22 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>347.25</v>
+        <v>358.75</v>
       </c>
       <c r="E37" s="1" t="inlineStr">
         <is>
-          <t>06-03-2026</t>
+          <t>11-03-2026</t>
         </is>
       </c>
       <c r="F37" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
@@ -1487,22 +1487,22 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>339.45</v>
+        <v>347.25</v>
       </c>
       <c r="E38" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>06-03-2026</t>
         </is>
       </c>
       <c r="F38" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
@@ -1515,22 +1515,22 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>330.95</v>
+        <v>339.45</v>
       </c>
       <c r="E39" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F39" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B40" s="1" t="inlineStr">
         <is>
@@ -1543,22 +1543,22 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>323.05</v>
+        <v>330.95</v>
       </c>
       <c r="E40" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="F40" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B41" s="1" t="inlineStr">
         <is>
@@ -1571,22 +1571,22 @@
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>316.15</v>
+        <v>323.05</v>
       </c>
       <c r="E41" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="F41" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B42" s="1" t="inlineStr">
         <is>
@@ -1599,22 +1599,22 @@
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>323.75</v>
+        <v>316.15</v>
       </c>
       <c r="E42" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="F42" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B43" s="1" t="inlineStr">
         <is>
@@ -1627,22 +1627,22 @@
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>318.05</v>
+        <v>323.75</v>
       </c>
       <c r="E43" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="F43" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B44" s="1" t="inlineStr">
         <is>
@@ -1655,22 +1655,22 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>320.45</v>
+        <v>318.05</v>
       </c>
       <c r="E44" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="F44" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B45" s="1" t="inlineStr">
         <is>
@@ -1683,22 +1683,22 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E45" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F45" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B46" s="1" t="inlineStr">
         <is>
@@ -1711,22 +1711,22 @@
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E46" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F46" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="B47" s="1" t="inlineStr">
         <is>
@@ -1739,22 +1739,22 @@
         </is>
       </c>
       <c r="D47" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E47" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F47" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B48" s="1" t="inlineStr">
         <is>
@@ -1767,22 +1767,22 @@
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E48" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F48" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B49" s="1" t="inlineStr">
         <is>
@@ -1795,22 +1795,22 @@
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>307.25</v>
+        <v>320.05</v>
       </c>
       <c r="E49" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="F49" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B50" s="1" t="inlineStr">
         <is>
@@ -1823,22 +1823,22 @@
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>301.65</v>
+        <v>307.25</v>
       </c>
       <c r="E50" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F50" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B51" s="1" t="inlineStr">
         <is>
@@ -1851,22 +1851,22 @@
         </is>
       </c>
       <c r="D51" s="2" t="n">
-        <v>296.05</v>
+        <v>301.65</v>
       </c>
       <c r="E51" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="F51" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B52" s="1" t="inlineStr">
         <is>
@@ -1879,22 +1879,22 @@
         </is>
       </c>
       <c r="D52" s="2" t="n">
-        <v>290.95</v>
+        <v>296.05</v>
       </c>
       <c r="E52" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="F52" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B53" s="1" t="inlineStr">
         <is>
@@ -1907,22 +1907,22 @@
         </is>
       </c>
       <c r="D53" s="2" t="n">
-        <v>283.55</v>
+        <v>290.95</v>
       </c>
       <c r="E53" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="F53" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B54" s="1" t="inlineStr">
         <is>
@@ -1935,22 +1935,22 @@
         </is>
       </c>
       <c r="D54" s="2" t="n">
-        <v>281.95</v>
+        <v>283.55</v>
       </c>
       <c r="E54" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="F54" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B55" s="1" t="inlineStr">
         <is>
@@ -1963,22 +1963,22 @@
         </is>
       </c>
       <c r="D55" s="2" t="n">
-        <v>292.65</v>
+        <v>281.95</v>
       </c>
       <c r="E55" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="F55" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B56" s="1" t="inlineStr">
         <is>
@@ -1991,22 +1991,22 @@
         </is>
       </c>
       <c r="D56" s="2" t="n">
-        <v>296.05</v>
+        <v>292.65</v>
       </c>
       <c r="E56" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="F56" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B57" s="1" t="inlineStr">
         <is>
@@ -2019,22 +2019,22 @@
         </is>
       </c>
       <c r="D57" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E57" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F57" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B58" s="1" t="inlineStr">
         <is>
@@ -2047,22 +2047,22 @@
         </is>
       </c>
       <c r="D58" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E58" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F58" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B59" s="1" t="inlineStr">
         <is>
@@ -2075,22 +2075,22 @@
         </is>
       </c>
       <c r="D59" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E59" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F59" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B60" s="1" t="inlineStr">
         <is>
@@ -2103,22 +2103,22 @@
         </is>
       </c>
       <c r="D60" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E60" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F60" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B61" s="1" t="inlineStr">
         <is>
@@ -2131,22 +2131,22 @@
         </is>
       </c>
       <c r="D61" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E61" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F61" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B62" s="1" t="inlineStr">
         <is>
@@ -2159,22 +2159,22 @@
         </is>
       </c>
       <c r="D62" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E62" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F62" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="1" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B63" s="1" t="inlineStr">
         <is>
@@ -2187,22 +2187,22 @@
         </is>
       </c>
       <c r="D63" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E63" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F63" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="1" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B64" s="1" t="inlineStr">
         <is>
@@ -2215,22 +2215,22 @@
         </is>
       </c>
       <c r="D64" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E64" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F64" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="1" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B65" s="1" t="inlineStr">
         <is>
@@ -2243,22 +2243,22 @@
         </is>
       </c>
       <c r="D65" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E65" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F65" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="1" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B66" s="1" t="inlineStr">
         <is>
@@ -2271,22 +2271,22 @@
         </is>
       </c>
       <c r="D66" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E66" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F66" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="1" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B67" s="1" t="inlineStr">
         <is>
@@ -2299,22 +2299,22 @@
         </is>
       </c>
       <c r="D67" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E67" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F67" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B68" s="1" t="inlineStr">
         <is>
@@ -2327,22 +2327,22 @@
         </is>
       </c>
       <c r="D68" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E68" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F68" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B69" s="1" t="inlineStr">
         <is>
@@ -2355,22 +2355,22 @@
         </is>
       </c>
       <c r="D69" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E69" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F69" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="1" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B70" s="1" t="inlineStr">
         <is>
@@ -2383,22 +2383,22 @@
         </is>
       </c>
       <c r="D70" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E70" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F70" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B71" s="1" t="inlineStr">
         <is>
@@ -2411,42 +2411,70 @@
         </is>
       </c>
       <c r="D71" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E71" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F71" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B72" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C72" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="n">
+        <v>269.45</v>
+      </c>
+      <c r="E72" s="1" t="inlineStr">
+        <is>
+          <t>15-08-2025</t>
+        </is>
+      </c>
+      <c r="F72" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B72" s="1" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C72" s="1" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D72" s="2" t="n">
+      <c r="B73" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C73" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="n">
         <v>268.25</v>
       </c>
-      <c r="E72" s="1" t="inlineStr">
+      <c r="E73" s="1" t="inlineStr">
         <is>
           <t>07-08-2025</t>
         </is>
       </c>
-      <c r="F72" s="1" t="inlineStr">
+      <c r="F73" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
@@ -2525,6 +2553,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F70" r:id="rId69"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F71" r:id="rId70"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F72" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F73" r:id="rId72"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-09-24 08:37:28 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F73"/>
+  <dimension ref="A1:F74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -466,7 +466,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -479,22 +479,22 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>367.65</v>
+        <v>362.75</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>19-09-2026</t>
+          <t>24-09-2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-09-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-09-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
@@ -507,22 +507,22 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>365.55</v>
+        <v>367.65</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>16-09-2026</t>
+          <t>19-09-2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-09-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-09-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
@@ -535,22 +535,22 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>371.55</v>
+        <v>365.55</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>11-09-2026</t>
+          <t>16-09-2026</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-09-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-09-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
@@ -563,22 +563,22 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>365.25</v>
+        <v>371.55</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>08-09-2026</t>
+          <t>11-09-2026</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-8-9-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-09-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
@@ -591,22 +591,22 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>361.65</v>
+        <v>365.25</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>02-09-2026</t>
+          <t>08-09-2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2026/09/Ingot-01-09-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-8-9-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
@@ -619,22 +619,22 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>360.15</v>
+        <v>361.65</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>28-08-2026</t>
+          <t>02-09-2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-08-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/09/Ingot-01-09-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
@@ -647,22 +647,22 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>356.25</v>
+        <v>360.15</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>21-08-2026</t>
+          <t>28-08-2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-21-08-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-08-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
@@ -675,22 +675,22 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>362.35</v>
+        <v>356.25</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>15-08-2026</t>
+          <t>21-08-2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-15-08-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-21-08-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
@@ -703,22 +703,22 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>375.25</v>
+        <v>362.35</v>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>12-08-2026</t>
+          <t>15-08-2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-12-08-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-15-08-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
@@ -731,22 +731,22 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>363.35</v>
+        <v>375.25</v>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>01-08-2026</t>
+          <t>12-08-2026</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-08-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-12-08-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
@@ -759,22 +759,22 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>354.95</v>
+        <v>363.35</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>29-07-2026</t>
+          <t>01-08-2026</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-08-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
@@ -787,22 +787,22 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>361.15</v>
+        <v>354.95</v>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>24-07-2026</t>
+          <t>29-07-2026</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-07-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
@@ -815,22 +815,22 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>356.35</v>
+        <v>361.15</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>18-07-2026</t>
+          <t>24-07-2026</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-07-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
@@ -843,22 +843,22 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>352.85</v>
+        <v>356.35</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>11-07-2026</t>
+          <t>18-07-2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
@@ -871,22 +871,22 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>349.05</v>
+        <v>352.85</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>08-07-2026</t>
+          <t>11-07-2026</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-08-07-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
@@ -899,22 +899,22 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>344.05</v>
+        <v>349.05</v>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>01-07-2026</t>
+          <t>08-07-2026</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-08-07-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
@@ -927,22 +927,22 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>349.05</v>
+        <v>344.05</v>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>29-06-2026</t>
+          <t>01-07-2026</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
@@ -959,18 +959,18 @@
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>26-06-2026</t>
+          <t>29-06-2026</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
@@ -983,22 +983,22 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>376.55</v>
+        <v>349.05</v>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>18-06-2026</t>
+          <t>26-06-2026</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
@@ -1026,7 +1026,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
@@ -1039,22 +1039,22 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>393.85</v>
+        <v>376.55</v>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>13-06-2026</t>
+          <t>18-06-2026</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
@@ -1067,22 +1067,22 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>402.35</v>
+        <v>393.85</v>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>10-06-2026</t>
+          <t>13-06-2026</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-10-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
@@ -1095,22 +1095,22 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>416.35</v>
+        <v>402.35</v>
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>05-06-2026</t>
+          <t>10-06-2026</t>
         </is>
       </c>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-10-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
@@ -1123,22 +1123,22 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>412.55</v>
+        <v>416.35</v>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>01-06-2026</t>
+          <t>05-06-2026</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
@@ -1151,22 +1151,22 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>411.05</v>
+        <v>412.55</v>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>27-05-2026</t>
+          <t>01-06-2026</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
@@ -1179,22 +1179,22 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>404.95</v>
+        <v>411.05</v>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>20-05-2026</t>
+          <t>27-05-2026</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
@@ -1207,22 +1207,22 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>408.85</v>
+        <v>404.95</v>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>14-05-2026</t>
+          <t>20-05-2026</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
@@ -1235,22 +1235,22 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>390.05</v>
+        <v>408.85</v>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>01-05-2026</t>
+          <t>14-05-2026</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
@@ -1263,22 +1263,22 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>392.55</v>
+        <v>390.05</v>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>24-04-2026</t>
+          <t>01-05-2026</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
@@ -1291,22 +1291,22 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>383.65</v>
+        <v>392.55</v>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>16-04-2026</t>
+          <t>24-04-2026</t>
         </is>
       </c>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
@@ -1319,22 +1319,22 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>373.55</v>
+        <v>383.65</v>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>03-04-2026</t>
+          <t>16-04-2026</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
@@ -1347,22 +1347,22 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>357.05</v>
+        <v>373.55</v>
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>28-03-2026</t>
+          <t>03-04-2026</t>
         </is>
       </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
@@ -1375,22 +1375,22 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>350.45</v>
+        <v>357.05</v>
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>24-03-2026</t>
+          <t>28-03-2026</t>
         </is>
       </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
@@ -1403,22 +1403,22 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>360.05</v>
+        <v>350.45</v>
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>19-03-2026</t>
+          <t>24-03-2026</t>
         </is>
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
@@ -1431,22 +1431,22 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>372.05</v>
+        <v>360.05</v>
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>14-03-2026</t>
+          <t>19-03-2026</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
@@ -1459,22 +1459,22 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>358.75</v>
+        <v>372.05</v>
       </c>
       <c r="E37" s="1" t="inlineStr">
         <is>
-          <t>11-03-2026</t>
+          <t>14-03-2026</t>
         </is>
       </c>
       <c r="F37" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
@@ -1487,22 +1487,22 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>347.25</v>
+        <v>358.75</v>
       </c>
       <c r="E38" s="1" t="inlineStr">
         <is>
-          <t>06-03-2026</t>
+          <t>11-03-2026</t>
         </is>
       </c>
       <c r="F38" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
@@ -1515,22 +1515,22 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>339.45</v>
+        <v>347.25</v>
       </c>
       <c r="E39" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>06-03-2026</t>
         </is>
       </c>
       <c r="F39" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B40" s="1" t="inlineStr">
         <is>
@@ -1543,22 +1543,22 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>330.95</v>
+        <v>339.45</v>
       </c>
       <c r="E40" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F40" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B41" s="1" t="inlineStr">
         <is>
@@ -1571,22 +1571,22 @@
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>323.05</v>
+        <v>330.95</v>
       </c>
       <c r="E41" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="F41" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B42" s="1" t="inlineStr">
         <is>
@@ -1599,22 +1599,22 @@
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>316.15</v>
+        <v>323.05</v>
       </c>
       <c r="E42" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="F42" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B43" s="1" t="inlineStr">
         <is>
@@ -1627,22 +1627,22 @@
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>323.75</v>
+        <v>316.15</v>
       </c>
       <c r="E43" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="F43" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B44" s="1" t="inlineStr">
         <is>
@@ -1655,22 +1655,22 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>318.05</v>
+        <v>323.75</v>
       </c>
       <c r="E44" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="F44" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B45" s="1" t="inlineStr">
         <is>
@@ -1683,22 +1683,22 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>320.45</v>
+        <v>318.05</v>
       </c>
       <c r="E45" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="F45" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B46" s="1" t="inlineStr">
         <is>
@@ -1711,22 +1711,22 @@
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E46" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F46" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B47" s="1" t="inlineStr">
         <is>
@@ -1739,22 +1739,22 @@
         </is>
       </c>
       <c r="D47" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E47" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F47" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="B48" s="1" t="inlineStr">
         <is>
@@ -1767,22 +1767,22 @@
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E48" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F48" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B49" s="1" t="inlineStr">
         <is>
@@ -1795,22 +1795,22 @@
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E49" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F49" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B50" s="1" t="inlineStr">
         <is>
@@ -1823,22 +1823,22 @@
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>307.25</v>
+        <v>320.05</v>
       </c>
       <c r="E50" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="F50" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B51" s="1" t="inlineStr">
         <is>
@@ -1851,22 +1851,22 @@
         </is>
       </c>
       <c r="D51" s="2" t="n">
-        <v>301.65</v>
+        <v>307.25</v>
       </c>
       <c r="E51" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F51" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B52" s="1" t="inlineStr">
         <is>
@@ -1879,22 +1879,22 @@
         </is>
       </c>
       <c r="D52" s="2" t="n">
-        <v>296.05</v>
+        <v>301.65</v>
       </c>
       <c r="E52" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="F52" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B53" s="1" t="inlineStr">
         <is>
@@ -1907,22 +1907,22 @@
         </is>
       </c>
       <c r="D53" s="2" t="n">
-        <v>290.95</v>
+        <v>296.05</v>
       </c>
       <c r="E53" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="F53" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B54" s="1" t="inlineStr">
         <is>
@@ -1935,22 +1935,22 @@
         </is>
       </c>
       <c r="D54" s="2" t="n">
-        <v>283.55</v>
+        <v>290.95</v>
       </c>
       <c r="E54" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="F54" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B55" s="1" t="inlineStr">
         <is>
@@ -1963,22 +1963,22 @@
         </is>
       </c>
       <c r="D55" s="2" t="n">
-        <v>281.95</v>
+        <v>283.55</v>
       </c>
       <c r="E55" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="F55" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B56" s="1" t="inlineStr">
         <is>
@@ -1991,22 +1991,22 @@
         </is>
       </c>
       <c r="D56" s="2" t="n">
-        <v>292.65</v>
+        <v>281.95</v>
       </c>
       <c r="E56" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="F56" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B57" s="1" t="inlineStr">
         <is>
@@ -2019,22 +2019,22 @@
         </is>
       </c>
       <c r="D57" s="2" t="n">
-        <v>296.05</v>
+        <v>292.65</v>
       </c>
       <c r="E57" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="F57" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B58" s="1" t="inlineStr">
         <is>
@@ -2047,22 +2047,22 @@
         </is>
       </c>
       <c r="D58" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E58" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F58" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B59" s="1" t="inlineStr">
         <is>
@@ -2075,22 +2075,22 @@
         </is>
       </c>
       <c r="D59" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E59" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F59" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B60" s="1" t="inlineStr">
         <is>
@@ -2103,22 +2103,22 @@
         </is>
       </c>
       <c r="D60" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E60" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F60" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B61" s="1" t="inlineStr">
         <is>
@@ -2131,22 +2131,22 @@
         </is>
       </c>
       <c r="D61" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E61" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F61" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B62" s="1" t="inlineStr">
         <is>
@@ -2159,22 +2159,22 @@
         </is>
       </c>
       <c r="D62" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E62" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F62" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="1" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B63" s="1" t="inlineStr">
         <is>
@@ -2187,22 +2187,22 @@
         </is>
       </c>
       <c r="D63" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E63" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F63" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="1" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B64" s="1" t="inlineStr">
         <is>
@@ -2215,22 +2215,22 @@
         </is>
       </c>
       <c r="D64" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E64" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F64" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="1" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B65" s="1" t="inlineStr">
         <is>
@@ -2243,22 +2243,22 @@
         </is>
       </c>
       <c r="D65" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E65" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F65" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="1" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B66" s="1" t="inlineStr">
         <is>
@@ -2271,22 +2271,22 @@
         </is>
       </c>
       <c r="D66" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E66" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F66" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="1" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B67" s="1" t="inlineStr">
         <is>
@@ -2299,22 +2299,22 @@
         </is>
       </c>
       <c r="D67" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E67" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F67" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="1" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B68" s="1" t="inlineStr">
         <is>
@@ -2327,22 +2327,22 @@
         </is>
       </c>
       <c r="D68" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E68" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F68" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B69" s="1" t="inlineStr">
         <is>
@@ -2355,22 +2355,22 @@
         </is>
       </c>
       <c r="D69" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E69" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F69" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B70" s="1" t="inlineStr">
         <is>
@@ -2383,22 +2383,22 @@
         </is>
       </c>
       <c r="D70" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E70" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F70" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="1" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B71" s="1" t="inlineStr">
         <is>
@@ -2411,22 +2411,22 @@
         </is>
       </c>
       <c r="D71" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E71" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F71" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B72" s="1" t="inlineStr">
         <is>
@@ -2439,42 +2439,70 @@
         </is>
       </c>
       <c r="D72" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E72" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F72" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B73" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C73" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="n">
+        <v>269.45</v>
+      </c>
+      <c r="E73" s="1" t="inlineStr">
+        <is>
+          <t>15-08-2025</t>
+        </is>
+      </c>
+      <c r="F73" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B73" s="1" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C73" s="1" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D73" s="2" t="n">
+      <c r="B74" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C74" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="n">
         <v>268.25</v>
       </c>
-      <c r="E73" s="1" t="inlineStr">
+      <c r="E74" s="1" t="inlineStr">
         <is>
           <t>07-08-2025</t>
         </is>
       </c>
-      <c r="F73" s="1" t="inlineStr">
+      <c r="F74" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
@@ -2554,6 +2582,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F71" r:id="rId70"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F72" r:id="rId71"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F73" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F74" r:id="rId73"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-02 09:57:29 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F74"/>
+  <dimension ref="A1:F75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -466,7 +466,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -479,22 +479,22 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>362.75</v>
+        <v>351.25</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>24-09-2026</t>
+          <t>01-10-2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-09-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
@@ -507,22 +507,22 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>367.65</v>
+        <v>362.75</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>19-09-2026</t>
+          <t>24-09-2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-09-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-09-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
@@ -535,22 +535,22 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>365.55</v>
+        <v>367.65</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>16-09-2026</t>
+          <t>19-09-2026</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-09-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-09-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
@@ -563,22 +563,22 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>371.55</v>
+        <v>365.55</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>11-09-2026</t>
+          <t>16-09-2026</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-09-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-09-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
@@ -591,22 +591,22 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>365.25</v>
+        <v>371.55</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>08-09-2026</t>
+          <t>11-09-2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-8-9-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-09-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
@@ -619,22 +619,22 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>361.65</v>
+        <v>365.25</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>02-09-2026</t>
+          <t>08-09-2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2026/09/Ingot-01-09-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-8-9-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
@@ -647,22 +647,22 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>360.15</v>
+        <v>361.65</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>28-08-2026</t>
+          <t>02-09-2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-08-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/09/Ingot-01-09-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
@@ -675,22 +675,22 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>356.25</v>
+        <v>360.15</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>21-08-2026</t>
+          <t>28-08-2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-21-08-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-08-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
@@ -703,22 +703,22 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>362.35</v>
+        <v>356.25</v>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>15-08-2026</t>
+          <t>21-08-2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-15-08-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-21-08-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
@@ -731,22 +731,22 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>375.25</v>
+        <v>362.35</v>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>12-08-2026</t>
+          <t>15-08-2026</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-12-08-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-15-08-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
@@ -759,22 +759,22 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>363.35</v>
+        <v>375.25</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>01-08-2026</t>
+          <t>12-08-2026</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-08-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-12-08-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
@@ -787,22 +787,22 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>354.95</v>
+        <v>363.35</v>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>29-07-2026</t>
+          <t>01-08-2026</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-08-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
@@ -815,22 +815,22 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>361.15</v>
+        <v>354.95</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>24-07-2026</t>
+          <t>29-07-2026</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-07-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
@@ -843,22 +843,22 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>356.35</v>
+        <v>361.15</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>18-07-2026</t>
+          <t>24-07-2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-07-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
@@ -871,22 +871,22 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>352.85</v>
+        <v>356.35</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>11-07-2026</t>
+          <t>18-07-2026</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
@@ -899,22 +899,22 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>349.05</v>
+        <v>352.85</v>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>08-07-2026</t>
+          <t>11-07-2026</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-08-07-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
@@ -927,22 +927,22 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>344.05</v>
+        <v>349.05</v>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>01-07-2026</t>
+          <t>08-07-2026</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-08-07-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
@@ -955,22 +955,22 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>349.05</v>
+        <v>344.05</v>
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>29-06-2026</t>
+          <t>01-07-2026</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
@@ -987,18 +987,18 @@
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>26-06-2026</t>
+          <t>29-06-2026</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
@@ -1011,22 +1011,22 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>376.55</v>
+        <v>349.05</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>18-06-2026</t>
+          <t>26-06-2026</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
@@ -1054,7 +1054,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
@@ -1067,22 +1067,22 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>393.85</v>
+        <v>376.55</v>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>13-06-2026</t>
+          <t>18-06-2026</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
@@ -1095,22 +1095,22 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>402.35</v>
+        <v>393.85</v>
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>10-06-2026</t>
+          <t>13-06-2026</t>
         </is>
       </c>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-10-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
@@ -1123,22 +1123,22 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>416.35</v>
+        <v>402.35</v>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>05-06-2026</t>
+          <t>10-06-2026</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-10-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
@@ -1151,22 +1151,22 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>412.55</v>
+        <v>416.35</v>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>01-06-2026</t>
+          <t>05-06-2026</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
@@ -1179,22 +1179,22 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>411.05</v>
+        <v>412.55</v>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>27-05-2026</t>
+          <t>01-06-2026</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
@@ -1207,22 +1207,22 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>404.95</v>
+        <v>411.05</v>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>20-05-2026</t>
+          <t>27-05-2026</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
@@ -1235,22 +1235,22 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>408.85</v>
+        <v>404.95</v>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>14-05-2026</t>
+          <t>20-05-2026</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
@@ -1263,22 +1263,22 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>390.05</v>
+        <v>408.85</v>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>01-05-2026</t>
+          <t>14-05-2026</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
@@ -1291,22 +1291,22 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>392.55</v>
+        <v>390.05</v>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>24-04-2026</t>
+          <t>01-05-2026</t>
         </is>
       </c>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
@@ -1319,22 +1319,22 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>383.65</v>
+        <v>392.55</v>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>16-04-2026</t>
+          <t>24-04-2026</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
@@ -1347,22 +1347,22 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>373.55</v>
+        <v>383.65</v>
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>03-04-2026</t>
+          <t>16-04-2026</t>
         </is>
       </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
@@ -1375,22 +1375,22 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>357.05</v>
+        <v>373.55</v>
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>28-03-2026</t>
+          <t>03-04-2026</t>
         </is>
       </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
@@ -1403,22 +1403,22 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>350.45</v>
+        <v>357.05</v>
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>24-03-2026</t>
+          <t>28-03-2026</t>
         </is>
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
@@ -1431,22 +1431,22 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>360.05</v>
+        <v>350.45</v>
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>19-03-2026</t>
+          <t>24-03-2026</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
@@ -1459,22 +1459,22 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>372.05</v>
+        <v>360.05</v>
       </c>
       <c r="E37" s="1" t="inlineStr">
         <is>
-          <t>14-03-2026</t>
+          <t>19-03-2026</t>
         </is>
       </c>
       <c r="F37" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
@@ -1487,22 +1487,22 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>358.75</v>
+        <v>372.05</v>
       </c>
       <c r="E38" s="1" t="inlineStr">
         <is>
-          <t>11-03-2026</t>
+          <t>14-03-2026</t>
         </is>
       </c>
       <c r="F38" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
@@ -1515,22 +1515,22 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>347.25</v>
+        <v>358.75</v>
       </c>
       <c r="E39" s="1" t="inlineStr">
         <is>
-          <t>06-03-2026</t>
+          <t>11-03-2026</t>
         </is>
       </c>
       <c r="F39" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B40" s="1" t="inlineStr">
         <is>
@@ -1543,22 +1543,22 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>339.45</v>
+        <v>347.25</v>
       </c>
       <c r="E40" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>06-03-2026</t>
         </is>
       </c>
       <c r="F40" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B41" s="1" t="inlineStr">
         <is>
@@ -1571,22 +1571,22 @@
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>330.95</v>
+        <v>339.45</v>
       </c>
       <c r="E41" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F41" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B42" s="1" t="inlineStr">
         <is>
@@ -1599,22 +1599,22 @@
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>323.05</v>
+        <v>330.95</v>
       </c>
       <c r="E42" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="F42" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B43" s="1" t="inlineStr">
         <is>
@@ -1627,22 +1627,22 @@
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>316.15</v>
+        <v>323.05</v>
       </c>
       <c r="E43" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="F43" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B44" s="1" t="inlineStr">
         <is>
@@ -1655,22 +1655,22 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>323.75</v>
+        <v>316.15</v>
       </c>
       <c r="E44" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="F44" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B45" s="1" t="inlineStr">
         <is>
@@ -1683,22 +1683,22 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>318.05</v>
+        <v>323.75</v>
       </c>
       <c r="E45" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="F45" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B46" s="1" t="inlineStr">
         <is>
@@ -1711,22 +1711,22 @@
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>320.45</v>
+        <v>318.05</v>
       </c>
       <c r="E46" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="F46" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B47" s="1" t="inlineStr">
         <is>
@@ -1739,22 +1739,22 @@
         </is>
       </c>
       <c r="D47" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E47" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F47" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B48" s="1" t="inlineStr">
         <is>
@@ -1767,22 +1767,22 @@
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E48" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F48" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="B49" s="1" t="inlineStr">
         <is>
@@ -1795,22 +1795,22 @@
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E49" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F49" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B50" s="1" t="inlineStr">
         <is>
@@ -1823,22 +1823,22 @@
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E50" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F50" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B51" s="1" t="inlineStr">
         <is>
@@ -1851,22 +1851,22 @@
         </is>
       </c>
       <c r="D51" s="2" t="n">
-        <v>307.25</v>
+        <v>320.05</v>
       </c>
       <c r="E51" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="F51" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B52" s="1" t="inlineStr">
         <is>
@@ -1879,22 +1879,22 @@
         </is>
       </c>
       <c r="D52" s="2" t="n">
-        <v>301.65</v>
+        <v>307.25</v>
       </c>
       <c r="E52" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F52" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B53" s="1" t="inlineStr">
         <is>
@@ -1907,22 +1907,22 @@
         </is>
       </c>
       <c r="D53" s="2" t="n">
-        <v>296.05</v>
+        <v>301.65</v>
       </c>
       <c r="E53" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="F53" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B54" s="1" t="inlineStr">
         <is>
@@ -1935,22 +1935,22 @@
         </is>
       </c>
       <c r="D54" s="2" t="n">
-        <v>290.95</v>
+        <v>296.05</v>
       </c>
       <c r="E54" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="F54" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B55" s="1" t="inlineStr">
         <is>
@@ -1963,22 +1963,22 @@
         </is>
       </c>
       <c r="D55" s="2" t="n">
-        <v>283.55</v>
+        <v>290.95</v>
       </c>
       <c r="E55" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="F55" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B56" s="1" t="inlineStr">
         <is>
@@ -1991,22 +1991,22 @@
         </is>
       </c>
       <c r="D56" s="2" t="n">
-        <v>281.95</v>
+        <v>283.55</v>
       </c>
       <c r="E56" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="F56" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B57" s="1" t="inlineStr">
         <is>
@@ -2019,22 +2019,22 @@
         </is>
       </c>
       <c r="D57" s="2" t="n">
-        <v>292.65</v>
+        <v>281.95</v>
       </c>
       <c r="E57" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="F57" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B58" s="1" t="inlineStr">
         <is>
@@ -2047,22 +2047,22 @@
         </is>
       </c>
       <c r="D58" s="2" t="n">
-        <v>296.05</v>
+        <v>292.65</v>
       </c>
       <c r="E58" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="F58" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B59" s="1" t="inlineStr">
         <is>
@@ -2075,22 +2075,22 @@
         </is>
       </c>
       <c r="D59" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E59" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F59" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B60" s="1" t="inlineStr">
         <is>
@@ -2103,22 +2103,22 @@
         </is>
       </c>
       <c r="D60" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E60" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F60" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B61" s="1" t="inlineStr">
         <is>
@@ -2131,22 +2131,22 @@
         </is>
       </c>
       <c r="D61" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E61" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F61" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B62" s="1" t="inlineStr">
         <is>
@@ -2159,22 +2159,22 @@
         </is>
       </c>
       <c r="D62" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E62" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F62" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="1" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B63" s="1" t="inlineStr">
         <is>
@@ -2187,22 +2187,22 @@
         </is>
       </c>
       <c r="D63" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E63" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F63" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="1" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B64" s="1" t="inlineStr">
         <is>
@@ -2215,22 +2215,22 @@
         </is>
       </c>
       <c r="D64" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E64" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F64" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="1" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B65" s="1" t="inlineStr">
         <is>
@@ -2243,22 +2243,22 @@
         </is>
       </c>
       <c r="D65" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E65" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F65" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="1" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B66" s="1" t="inlineStr">
         <is>
@@ -2271,22 +2271,22 @@
         </is>
       </c>
       <c r="D66" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E66" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F66" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="1" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B67" s="1" t="inlineStr">
         <is>
@@ -2299,22 +2299,22 @@
         </is>
       </c>
       <c r="D67" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E67" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F67" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="1" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B68" s="1" t="inlineStr">
         <is>
@@ -2327,22 +2327,22 @@
         </is>
       </c>
       <c r="D68" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E68" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F68" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="1" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B69" s="1" t="inlineStr">
         <is>
@@ -2355,22 +2355,22 @@
         </is>
       </c>
       <c r="D69" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E69" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F69" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B70" s="1" t="inlineStr">
         <is>
@@ -2383,22 +2383,22 @@
         </is>
       </c>
       <c r="D70" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E70" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F70" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B71" s="1" t="inlineStr">
         <is>
@@ -2411,22 +2411,22 @@
         </is>
       </c>
       <c r="D71" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E71" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F71" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="1" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B72" s="1" t="inlineStr">
         <is>
@@ -2439,22 +2439,22 @@
         </is>
       </c>
       <c r="D72" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E72" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F72" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B73" s="1" t="inlineStr">
         <is>
@@ -2467,42 +2467,70 @@
         </is>
       </c>
       <c r="D73" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E73" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F73" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B74" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C74" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="n">
+        <v>269.45</v>
+      </c>
+      <c r="E74" s="1" t="inlineStr">
+        <is>
+          <t>15-08-2025</t>
+        </is>
+      </c>
+      <c r="F74" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B74" s="1" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C74" s="1" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D74" s="2" t="n">
+      <c r="B75" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C75" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="n">
         <v>268.25</v>
       </c>
-      <c r="E74" s="1" t="inlineStr">
+      <c r="E75" s="1" t="inlineStr">
         <is>
           <t>07-08-2025</t>
         </is>
       </c>
-      <c r="F74" s="1" t="inlineStr">
+      <c r="F75" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
@@ -2583,6 +2611,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F72" r:id="rId71"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F73" r:id="rId72"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F74" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F75" r:id="rId74"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-13 10:51:50 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F75"/>
+  <dimension ref="A1:F76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -466,7 +466,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -479,22 +479,22 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>351.25</v>
+        <v>343.65</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>01-10-2026</t>
+          <t>13-10-2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-10-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
@@ -507,22 +507,22 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>362.75</v>
+        <v>351.25</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>24-09-2026</t>
+          <t>01-10-2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-09-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
@@ -535,22 +535,22 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>367.65</v>
+        <v>362.75</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>19-09-2026</t>
+          <t>24-09-2026</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-09-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-09-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
@@ -563,22 +563,22 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>365.55</v>
+        <v>367.65</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>16-09-2026</t>
+          <t>19-09-2026</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-09-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-09-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
@@ -591,22 +591,22 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>371.55</v>
+        <v>365.55</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>11-09-2026</t>
+          <t>16-09-2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-09-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-09-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
@@ -619,22 +619,22 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>365.25</v>
+        <v>371.55</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>08-09-2026</t>
+          <t>11-09-2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-8-9-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-09-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
@@ -647,22 +647,22 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>361.65</v>
+        <v>365.25</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>02-09-2026</t>
+          <t>08-09-2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2026/09/Ingot-01-09-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-8-9-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
@@ -675,22 +675,22 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>360.15</v>
+        <v>361.65</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>28-08-2026</t>
+          <t>02-09-2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-08-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/09/Ingot-01-09-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
@@ -703,22 +703,22 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>356.25</v>
+        <v>360.15</v>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>21-08-2026</t>
+          <t>28-08-2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-21-08-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-08-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
@@ -731,22 +731,22 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>362.35</v>
+        <v>356.25</v>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>15-08-2026</t>
+          <t>21-08-2026</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-15-08-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-21-08-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
@@ -759,22 +759,22 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>375.25</v>
+        <v>362.35</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>12-08-2026</t>
+          <t>15-08-2026</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-12-08-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-15-08-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
@@ -787,22 +787,22 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>363.35</v>
+        <v>375.25</v>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>01-08-2026</t>
+          <t>12-08-2026</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-08-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-12-08-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
@@ -815,22 +815,22 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>354.95</v>
+        <v>363.35</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>29-07-2026</t>
+          <t>01-08-2026</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-08-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
@@ -843,22 +843,22 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>361.15</v>
+        <v>354.95</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>24-07-2026</t>
+          <t>29-07-2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-07-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
@@ -871,22 +871,22 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>356.35</v>
+        <v>361.15</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>18-07-2026</t>
+          <t>24-07-2026</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-07-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
@@ -899,22 +899,22 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>352.85</v>
+        <v>356.35</v>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>11-07-2026</t>
+          <t>18-07-2026</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
@@ -927,22 +927,22 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>349.05</v>
+        <v>352.85</v>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>08-07-2026</t>
+          <t>11-07-2026</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-08-07-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
@@ -955,22 +955,22 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>344.05</v>
+        <v>349.05</v>
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>01-07-2026</t>
+          <t>08-07-2026</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-08-07-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
@@ -983,22 +983,22 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>349.05</v>
+        <v>344.05</v>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>29-06-2026</t>
+          <t>01-07-2026</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
@@ -1015,18 +1015,18 @@
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>26-06-2026</t>
+          <t>29-06-2026</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
@@ -1039,22 +1039,22 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>376.55</v>
+        <v>349.05</v>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>18-06-2026</t>
+          <t>26-06-2026</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
@@ -1082,7 +1082,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
@@ -1095,22 +1095,22 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>393.85</v>
+        <v>376.55</v>
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>13-06-2026</t>
+          <t>18-06-2026</t>
         </is>
       </c>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
@@ -1123,22 +1123,22 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>402.35</v>
+        <v>393.85</v>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>10-06-2026</t>
+          <t>13-06-2026</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-10-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
@@ -1151,22 +1151,22 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>416.35</v>
+        <v>402.35</v>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>05-06-2026</t>
+          <t>10-06-2026</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-10-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
@@ -1179,22 +1179,22 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>412.55</v>
+        <v>416.35</v>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>01-06-2026</t>
+          <t>05-06-2026</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
@@ -1207,22 +1207,22 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>411.05</v>
+        <v>412.55</v>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>27-05-2026</t>
+          <t>01-06-2026</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
@@ -1235,22 +1235,22 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>404.95</v>
+        <v>411.05</v>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>20-05-2026</t>
+          <t>27-05-2026</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
@@ -1263,22 +1263,22 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>408.85</v>
+        <v>404.95</v>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>14-05-2026</t>
+          <t>20-05-2026</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
@@ -1291,22 +1291,22 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>390.05</v>
+        <v>408.85</v>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>01-05-2026</t>
+          <t>14-05-2026</t>
         </is>
       </c>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
@@ -1319,22 +1319,22 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>392.55</v>
+        <v>390.05</v>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>24-04-2026</t>
+          <t>01-05-2026</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
@@ -1347,22 +1347,22 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>383.65</v>
+        <v>392.55</v>
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>16-04-2026</t>
+          <t>24-04-2026</t>
         </is>
       </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
@@ -1375,22 +1375,22 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>373.55</v>
+        <v>383.65</v>
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>03-04-2026</t>
+          <t>16-04-2026</t>
         </is>
       </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
@@ -1403,22 +1403,22 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>357.05</v>
+        <v>373.55</v>
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>28-03-2026</t>
+          <t>03-04-2026</t>
         </is>
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
@@ -1431,22 +1431,22 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>350.45</v>
+        <v>357.05</v>
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>24-03-2026</t>
+          <t>28-03-2026</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
@@ -1459,22 +1459,22 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>360.05</v>
+        <v>350.45</v>
       </c>
       <c r="E37" s="1" t="inlineStr">
         <is>
-          <t>19-03-2026</t>
+          <t>24-03-2026</t>
         </is>
       </c>
       <c r="F37" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
@@ -1487,22 +1487,22 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>372.05</v>
+        <v>360.05</v>
       </c>
       <c r="E38" s="1" t="inlineStr">
         <is>
-          <t>14-03-2026</t>
+          <t>19-03-2026</t>
         </is>
       </c>
       <c r="F38" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
@@ -1515,22 +1515,22 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>358.75</v>
+        <v>372.05</v>
       </c>
       <c r="E39" s="1" t="inlineStr">
         <is>
-          <t>11-03-2026</t>
+          <t>14-03-2026</t>
         </is>
       </c>
       <c r="F39" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B40" s="1" t="inlineStr">
         <is>
@@ -1543,22 +1543,22 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>347.25</v>
+        <v>358.75</v>
       </c>
       <c r="E40" s="1" t="inlineStr">
         <is>
-          <t>06-03-2026</t>
+          <t>11-03-2026</t>
         </is>
       </c>
       <c r="F40" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B41" s="1" t="inlineStr">
         <is>
@@ -1571,22 +1571,22 @@
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>339.45</v>
+        <v>347.25</v>
       </c>
       <c r="E41" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>06-03-2026</t>
         </is>
       </c>
       <c r="F41" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B42" s="1" t="inlineStr">
         <is>
@@ -1599,22 +1599,22 @@
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>330.95</v>
+        <v>339.45</v>
       </c>
       <c r="E42" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F42" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B43" s="1" t="inlineStr">
         <is>
@@ -1627,22 +1627,22 @@
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>323.05</v>
+        <v>330.95</v>
       </c>
       <c r="E43" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="F43" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B44" s="1" t="inlineStr">
         <is>
@@ -1655,22 +1655,22 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>316.15</v>
+        <v>323.05</v>
       </c>
       <c r="E44" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="F44" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B45" s="1" t="inlineStr">
         <is>
@@ -1683,22 +1683,22 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>323.75</v>
+        <v>316.15</v>
       </c>
       <c r="E45" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="F45" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B46" s="1" t="inlineStr">
         <is>
@@ -1711,22 +1711,22 @@
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>318.05</v>
+        <v>323.75</v>
       </c>
       <c r="E46" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="F46" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B47" s="1" t="inlineStr">
         <is>
@@ -1739,22 +1739,22 @@
         </is>
       </c>
       <c r="D47" s="2" t="n">
-        <v>320.45</v>
+        <v>318.05</v>
       </c>
       <c r="E47" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="F47" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B48" s="1" t="inlineStr">
         <is>
@@ -1767,22 +1767,22 @@
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E48" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F48" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B49" s="1" t="inlineStr">
         <is>
@@ -1795,22 +1795,22 @@
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E49" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F49" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="B50" s="1" t="inlineStr">
         <is>
@@ -1823,22 +1823,22 @@
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E50" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F50" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B51" s="1" t="inlineStr">
         <is>
@@ -1851,22 +1851,22 @@
         </is>
       </c>
       <c r="D51" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E51" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F51" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B52" s="1" t="inlineStr">
         <is>
@@ -1879,22 +1879,22 @@
         </is>
       </c>
       <c r="D52" s="2" t="n">
-        <v>307.25</v>
+        <v>320.05</v>
       </c>
       <c r="E52" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="F52" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B53" s="1" t="inlineStr">
         <is>
@@ -1907,22 +1907,22 @@
         </is>
       </c>
       <c r="D53" s="2" t="n">
-        <v>301.65</v>
+        <v>307.25</v>
       </c>
       <c r="E53" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F53" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B54" s="1" t="inlineStr">
         <is>
@@ -1935,22 +1935,22 @@
         </is>
       </c>
       <c r="D54" s="2" t="n">
-        <v>296.05</v>
+        <v>301.65</v>
       </c>
       <c r="E54" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="F54" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B55" s="1" t="inlineStr">
         <is>
@@ -1963,22 +1963,22 @@
         </is>
       </c>
       <c r="D55" s="2" t="n">
-        <v>290.95</v>
+        <v>296.05</v>
       </c>
       <c r="E55" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="F55" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B56" s="1" t="inlineStr">
         <is>
@@ -1991,22 +1991,22 @@
         </is>
       </c>
       <c r="D56" s="2" t="n">
-        <v>283.55</v>
+        <v>290.95</v>
       </c>
       <c r="E56" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="F56" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B57" s="1" t="inlineStr">
         <is>
@@ -2019,22 +2019,22 @@
         </is>
       </c>
       <c r="D57" s="2" t="n">
-        <v>281.95</v>
+        <v>283.55</v>
       </c>
       <c r="E57" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="F57" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B58" s="1" t="inlineStr">
         <is>
@@ -2047,22 +2047,22 @@
         </is>
       </c>
       <c r="D58" s="2" t="n">
-        <v>292.65</v>
+        <v>281.95</v>
       </c>
       <c r="E58" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="F58" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B59" s="1" t="inlineStr">
         <is>
@@ -2075,22 +2075,22 @@
         </is>
       </c>
       <c r="D59" s="2" t="n">
-        <v>296.05</v>
+        <v>292.65</v>
       </c>
       <c r="E59" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="F59" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B60" s="1" t="inlineStr">
         <is>
@@ -2103,22 +2103,22 @@
         </is>
       </c>
       <c r="D60" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E60" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F60" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B61" s="1" t="inlineStr">
         <is>
@@ -2131,22 +2131,22 @@
         </is>
       </c>
       <c r="D61" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E61" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F61" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B62" s="1" t="inlineStr">
         <is>
@@ -2159,22 +2159,22 @@
         </is>
       </c>
       <c r="D62" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E62" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F62" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="1" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B63" s="1" t="inlineStr">
         <is>
@@ -2187,22 +2187,22 @@
         </is>
       </c>
       <c r="D63" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E63" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F63" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="1" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B64" s="1" t="inlineStr">
         <is>
@@ -2215,22 +2215,22 @@
         </is>
       </c>
       <c r="D64" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E64" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F64" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="1" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B65" s="1" t="inlineStr">
         <is>
@@ -2243,22 +2243,22 @@
         </is>
       </c>
       <c r="D65" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E65" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F65" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="1" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B66" s="1" t="inlineStr">
         <is>
@@ -2271,22 +2271,22 @@
         </is>
       </c>
       <c r="D66" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E66" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F66" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="1" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B67" s="1" t="inlineStr">
         <is>
@@ -2299,22 +2299,22 @@
         </is>
       </c>
       <c r="D67" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E67" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F67" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="1" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B68" s="1" t="inlineStr">
         <is>
@@ -2327,22 +2327,22 @@
         </is>
       </c>
       <c r="D68" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E68" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F68" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="1" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B69" s="1" t="inlineStr">
         <is>
@@ -2355,22 +2355,22 @@
         </is>
       </c>
       <c r="D69" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E69" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F69" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="1" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B70" s="1" t="inlineStr">
         <is>
@@ -2383,22 +2383,22 @@
         </is>
       </c>
       <c r="D70" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E70" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F70" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B71" s="1" t="inlineStr">
         <is>
@@ -2411,22 +2411,22 @@
         </is>
       </c>
       <c r="D71" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E71" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F71" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B72" s="1" t="inlineStr">
         <is>
@@ -2439,22 +2439,22 @@
         </is>
       </c>
       <c r="D72" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E72" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F72" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="1" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B73" s="1" t="inlineStr">
         <is>
@@ -2467,22 +2467,22 @@
         </is>
       </c>
       <c r="D73" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E73" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F73" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B74" s="1" t="inlineStr">
         <is>
@@ -2495,42 +2495,70 @@
         </is>
       </c>
       <c r="D74" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E74" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F74" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B75" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C75" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="n">
+        <v>269.45</v>
+      </c>
+      <c r="E75" s="1" t="inlineStr">
+        <is>
+          <t>15-08-2025</t>
+        </is>
+      </c>
+      <c r="F75" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B75" s="1" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C75" s="1" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D75" s="2" t="n">
+      <c r="B76" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C76" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="n">
         <v>268.25</v>
       </c>
-      <c r="E75" s="1" t="inlineStr">
+      <c r="E76" s="1" t="inlineStr">
         <is>
           <t>07-08-2025</t>
         </is>
       </c>
-      <c r="F75" s="1" t="inlineStr">
+      <c r="F76" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
@@ -2612,6 +2640,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F73" r:id="rId72"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F74" r:id="rId73"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F75" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F76" r:id="rId75"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-16 08:21:49 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F76"/>
+  <dimension ref="A1:F77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -466,7 +466,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -479,22 +479,22 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>343.65</v>
+        <v>335.75</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>13-10-2026</t>
+          <t>16-10-2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-10-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-10-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
@@ -507,22 +507,22 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>351.25</v>
+        <v>343.65</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>01-10-2026</t>
+          <t>13-10-2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-10-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
@@ -535,22 +535,22 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>362.75</v>
+        <v>351.25</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>24-09-2026</t>
+          <t>01-10-2026</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-09-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
@@ -563,22 +563,22 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>367.65</v>
+        <v>362.75</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>19-09-2026</t>
+          <t>24-09-2026</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-09-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-09-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
@@ -591,22 +591,22 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>365.55</v>
+        <v>367.65</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>16-09-2026</t>
+          <t>19-09-2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-09-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-09-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
@@ -619,22 +619,22 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>371.55</v>
+        <v>365.55</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>11-09-2026</t>
+          <t>16-09-2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-09-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-09-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
@@ -647,22 +647,22 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>365.25</v>
+        <v>371.55</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>08-09-2026</t>
+          <t>11-09-2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-8-9-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-09-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
@@ -675,22 +675,22 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>361.65</v>
+        <v>365.25</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>02-09-2026</t>
+          <t>08-09-2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2026/09/Ingot-01-09-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-8-9-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
@@ -703,22 +703,22 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>360.15</v>
+        <v>361.65</v>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>28-08-2026</t>
+          <t>02-09-2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-08-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/09/Ingot-01-09-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
@@ -731,22 +731,22 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>356.25</v>
+        <v>360.15</v>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>21-08-2026</t>
+          <t>28-08-2026</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-21-08-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-08-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
@@ -759,22 +759,22 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>362.35</v>
+        <v>356.25</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>15-08-2026</t>
+          <t>21-08-2026</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-15-08-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-21-08-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
@@ -787,22 +787,22 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>375.25</v>
+        <v>362.35</v>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>12-08-2026</t>
+          <t>15-08-2026</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-12-08-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-15-08-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
@@ -815,22 +815,22 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>363.35</v>
+        <v>375.25</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>01-08-2026</t>
+          <t>12-08-2026</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-08-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-12-08-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
@@ -843,22 +843,22 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>354.95</v>
+        <v>363.35</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>29-07-2026</t>
+          <t>01-08-2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-08-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
@@ -871,22 +871,22 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>361.15</v>
+        <v>354.95</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>24-07-2026</t>
+          <t>29-07-2026</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-07-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
@@ -899,22 +899,22 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>356.35</v>
+        <v>361.15</v>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>18-07-2026</t>
+          <t>24-07-2026</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-07-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
@@ -927,22 +927,22 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>352.85</v>
+        <v>356.35</v>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>11-07-2026</t>
+          <t>18-07-2026</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
@@ -955,22 +955,22 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>349.05</v>
+        <v>352.85</v>
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>08-07-2026</t>
+          <t>11-07-2026</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-08-07-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
@@ -983,22 +983,22 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>344.05</v>
+        <v>349.05</v>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>01-07-2026</t>
+          <t>08-07-2026</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-08-07-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
@@ -1011,22 +1011,22 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>349.05</v>
+        <v>344.05</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>29-06-2026</t>
+          <t>01-07-2026</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
@@ -1043,18 +1043,18 @@
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>26-06-2026</t>
+          <t>29-06-2026</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
@@ -1067,22 +1067,22 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>376.55</v>
+        <v>349.05</v>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>18-06-2026</t>
+          <t>26-06-2026</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
@@ -1110,7 +1110,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
@@ -1123,22 +1123,22 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>393.85</v>
+        <v>376.55</v>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>13-06-2026</t>
+          <t>18-06-2026</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
@@ -1151,22 +1151,22 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>402.35</v>
+        <v>393.85</v>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>10-06-2026</t>
+          <t>13-06-2026</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-10-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
@@ -1179,22 +1179,22 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>416.35</v>
+        <v>402.35</v>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>05-06-2026</t>
+          <t>10-06-2026</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-10-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
@@ -1207,22 +1207,22 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>412.55</v>
+        <v>416.35</v>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>01-06-2026</t>
+          <t>05-06-2026</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
@@ -1235,22 +1235,22 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>411.05</v>
+        <v>412.55</v>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>27-05-2026</t>
+          <t>01-06-2026</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
@@ -1263,22 +1263,22 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>404.95</v>
+        <v>411.05</v>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>20-05-2026</t>
+          <t>27-05-2026</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
@@ -1291,22 +1291,22 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>408.85</v>
+        <v>404.95</v>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>14-05-2026</t>
+          <t>20-05-2026</t>
         </is>
       </c>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
@@ -1319,22 +1319,22 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>390.05</v>
+        <v>408.85</v>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>01-05-2026</t>
+          <t>14-05-2026</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
@@ -1347,22 +1347,22 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>392.55</v>
+        <v>390.05</v>
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>24-04-2026</t>
+          <t>01-05-2026</t>
         </is>
       </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
@@ -1375,22 +1375,22 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>383.65</v>
+        <v>392.55</v>
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>16-04-2026</t>
+          <t>24-04-2026</t>
         </is>
       </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
@@ -1403,22 +1403,22 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>373.55</v>
+        <v>383.65</v>
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>03-04-2026</t>
+          <t>16-04-2026</t>
         </is>
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
@@ -1431,22 +1431,22 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>357.05</v>
+        <v>373.55</v>
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>28-03-2026</t>
+          <t>03-04-2026</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
@@ -1459,22 +1459,22 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>350.45</v>
+        <v>357.05</v>
       </c>
       <c r="E37" s="1" t="inlineStr">
         <is>
-          <t>24-03-2026</t>
+          <t>28-03-2026</t>
         </is>
       </c>
       <c r="F37" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
@@ -1487,22 +1487,22 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>360.05</v>
+        <v>350.45</v>
       </c>
       <c r="E38" s="1" t="inlineStr">
         <is>
-          <t>19-03-2026</t>
+          <t>24-03-2026</t>
         </is>
       </c>
       <c r="F38" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
@@ -1515,22 +1515,22 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>372.05</v>
+        <v>360.05</v>
       </c>
       <c r="E39" s="1" t="inlineStr">
         <is>
-          <t>14-03-2026</t>
+          <t>19-03-2026</t>
         </is>
       </c>
       <c r="F39" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B40" s="1" t="inlineStr">
         <is>
@@ -1543,22 +1543,22 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>358.75</v>
+        <v>372.05</v>
       </c>
       <c r="E40" s="1" t="inlineStr">
         <is>
-          <t>11-03-2026</t>
+          <t>14-03-2026</t>
         </is>
       </c>
       <c r="F40" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B41" s="1" t="inlineStr">
         <is>
@@ -1571,22 +1571,22 @@
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>347.25</v>
+        <v>358.75</v>
       </c>
       <c r="E41" s="1" t="inlineStr">
         <is>
-          <t>06-03-2026</t>
+          <t>11-03-2026</t>
         </is>
       </c>
       <c r="F41" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B42" s="1" t="inlineStr">
         <is>
@@ -1599,22 +1599,22 @@
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>339.45</v>
+        <v>347.25</v>
       </c>
       <c r="E42" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>06-03-2026</t>
         </is>
       </c>
       <c r="F42" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B43" s="1" t="inlineStr">
         <is>
@@ -1627,22 +1627,22 @@
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>330.95</v>
+        <v>339.45</v>
       </c>
       <c r="E43" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F43" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B44" s="1" t="inlineStr">
         <is>
@@ -1655,22 +1655,22 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>323.05</v>
+        <v>330.95</v>
       </c>
       <c r="E44" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="F44" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B45" s="1" t="inlineStr">
         <is>
@@ -1683,22 +1683,22 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>316.15</v>
+        <v>323.05</v>
       </c>
       <c r="E45" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="F45" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B46" s="1" t="inlineStr">
         <is>
@@ -1711,22 +1711,22 @@
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>323.75</v>
+        <v>316.15</v>
       </c>
       <c r="E46" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="F46" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B47" s="1" t="inlineStr">
         <is>
@@ -1739,22 +1739,22 @@
         </is>
       </c>
       <c r="D47" s="2" t="n">
-        <v>318.05</v>
+        <v>323.75</v>
       </c>
       <c r="E47" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="F47" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B48" s="1" t="inlineStr">
         <is>
@@ -1767,22 +1767,22 @@
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>320.45</v>
+        <v>318.05</v>
       </c>
       <c r="E48" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="F48" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B49" s="1" t="inlineStr">
         <is>
@@ -1795,22 +1795,22 @@
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E49" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F49" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B50" s="1" t="inlineStr">
         <is>
@@ -1823,22 +1823,22 @@
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E50" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F50" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="B51" s="1" t="inlineStr">
         <is>
@@ -1851,22 +1851,22 @@
         </is>
       </c>
       <c r="D51" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E51" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F51" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B52" s="1" t="inlineStr">
         <is>
@@ -1879,22 +1879,22 @@
         </is>
       </c>
       <c r="D52" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E52" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F52" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B53" s="1" t="inlineStr">
         <is>
@@ -1907,22 +1907,22 @@
         </is>
       </c>
       <c r="D53" s="2" t="n">
-        <v>307.25</v>
+        <v>320.05</v>
       </c>
       <c r="E53" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="F53" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B54" s="1" t="inlineStr">
         <is>
@@ -1935,22 +1935,22 @@
         </is>
       </c>
       <c r="D54" s="2" t="n">
-        <v>301.65</v>
+        <v>307.25</v>
       </c>
       <c r="E54" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F54" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B55" s="1" t="inlineStr">
         <is>
@@ -1963,22 +1963,22 @@
         </is>
       </c>
       <c r="D55" s="2" t="n">
-        <v>296.05</v>
+        <v>301.65</v>
       </c>
       <c r="E55" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="F55" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B56" s="1" t="inlineStr">
         <is>
@@ -1991,22 +1991,22 @@
         </is>
       </c>
       <c r="D56" s="2" t="n">
-        <v>290.95</v>
+        <v>296.05</v>
       </c>
       <c r="E56" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="F56" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B57" s="1" t="inlineStr">
         <is>
@@ -2019,22 +2019,22 @@
         </is>
       </c>
       <c r="D57" s="2" t="n">
-        <v>283.55</v>
+        <v>290.95</v>
       </c>
       <c r="E57" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="F57" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B58" s="1" t="inlineStr">
         <is>
@@ -2047,22 +2047,22 @@
         </is>
       </c>
       <c r="D58" s="2" t="n">
-        <v>281.95</v>
+        <v>283.55</v>
       </c>
       <c r="E58" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="F58" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B59" s="1" t="inlineStr">
         <is>
@@ -2075,22 +2075,22 @@
         </is>
       </c>
       <c r="D59" s="2" t="n">
-        <v>292.65</v>
+        <v>281.95</v>
       </c>
       <c r="E59" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="F59" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B60" s="1" t="inlineStr">
         <is>
@@ -2103,22 +2103,22 @@
         </is>
       </c>
       <c r="D60" s="2" t="n">
-        <v>296.05</v>
+        <v>292.65</v>
       </c>
       <c r="E60" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="F60" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B61" s="1" t="inlineStr">
         <is>
@@ -2131,22 +2131,22 @@
         </is>
       </c>
       <c r="D61" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E61" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F61" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B62" s="1" t="inlineStr">
         <is>
@@ -2159,22 +2159,22 @@
         </is>
       </c>
       <c r="D62" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E62" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F62" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="1" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B63" s="1" t="inlineStr">
         <is>
@@ -2187,22 +2187,22 @@
         </is>
       </c>
       <c r="D63" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E63" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F63" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="1" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B64" s="1" t="inlineStr">
         <is>
@@ -2215,22 +2215,22 @@
         </is>
       </c>
       <c r="D64" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E64" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F64" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="1" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B65" s="1" t="inlineStr">
         <is>
@@ -2243,22 +2243,22 @@
         </is>
       </c>
       <c r="D65" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E65" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F65" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="1" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B66" s="1" t="inlineStr">
         <is>
@@ -2271,22 +2271,22 @@
         </is>
       </c>
       <c r="D66" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E66" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F66" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="1" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B67" s="1" t="inlineStr">
         <is>
@@ -2299,22 +2299,22 @@
         </is>
       </c>
       <c r="D67" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E67" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F67" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="1" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B68" s="1" t="inlineStr">
         <is>
@@ -2327,22 +2327,22 @@
         </is>
       </c>
       <c r="D68" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E68" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F68" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="1" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B69" s="1" t="inlineStr">
         <is>
@@ -2355,22 +2355,22 @@
         </is>
       </c>
       <c r="D69" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E69" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F69" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="1" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B70" s="1" t="inlineStr">
         <is>
@@ -2383,22 +2383,22 @@
         </is>
       </c>
       <c r="D70" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E70" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F70" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="1" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B71" s="1" t="inlineStr">
         <is>
@@ -2411,22 +2411,22 @@
         </is>
       </c>
       <c r="D71" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E71" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F71" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B72" s="1" t="inlineStr">
         <is>
@@ -2439,22 +2439,22 @@
         </is>
       </c>
       <c r="D72" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E72" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F72" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B73" s="1" t="inlineStr">
         <is>
@@ -2467,22 +2467,22 @@
         </is>
       </c>
       <c r="D73" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E73" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F73" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="1" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B74" s="1" t="inlineStr">
         <is>
@@ -2495,22 +2495,22 @@
         </is>
       </c>
       <c r="D74" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E74" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F74" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B75" s="1" t="inlineStr">
         <is>
@@ -2523,42 +2523,70 @@
         </is>
       </c>
       <c r="D75" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E75" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F75" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B76" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C76" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="n">
+        <v>269.45</v>
+      </c>
+      <c r="E76" s="1" t="inlineStr">
+        <is>
+          <t>15-08-2025</t>
+        </is>
+      </c>
+      <c r="F76" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B76" s="1" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C76" s="1" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D76" s="2" t="n">
+      <c r="B77" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C77" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="n">
         <v>268.25</v>
       </c>
-      <c r="E76" s="1" t="inlineStr">
+      <c r="E77" s="1" t="inlineStr">
         <is>
           <t>07-08-2025</t>
         </is>
       </c>
-      <c r="F76" s="1" t="inlineStr">
+      <c r="F77" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
@@ -2641,6 +2669,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F74" r:id="rId73"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F75" r:id="rId74"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F76" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F77" r:id="rId76"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-24 08:18:14 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F77"/>
+  <dimension ref="A1:F78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -466,7 +466,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -479,22 +479,22 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>335.75</v>
+        <v>339.85</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>16-10-2026</t>
+          <t>24-10-2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-10-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-10-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
@@ -507,22 +507,22 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>343.65</v>
+        <v>335.75</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>13-10-2026</t>
+          <t>16-10-2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-10-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-10-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
@@ -535,22 +535,22 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>351.25</v>
+        <v>343.65</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>01-10-2026</t>
+          <t>13-10-2026</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-10-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
@@ -563,22 +563,22 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>362.75</v>
+        <v>351.25</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>24-09-2026</t>
+          <t>01-10-2026</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-09-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
@@ -591,22 +591,22 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>367.65</v>
+        <v>362.75</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>19-09-2026</t>
+          <t>24-09-2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-09-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-09-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
@@ -619,22 +619,22 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>365.55</v>
+        <v>367.65</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>16-09-2026</t>
+          <t>19-09-2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-09-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-09-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
@@ -647,22 +647,22 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>371.55</v>
+        <v>365.55</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>11-09-2026</t>
+          <t>16-09-2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-09-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-09-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
@@ -675,22 +675,22 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>365.25</v>
+        <v>371.55</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>08-09-2026</t>
+          <t>11-09-2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-8-9-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-09-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
@@ -703,22 +703,22 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>361.65</v>
+        <v>365.25</v>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>02-09-2026</t>
+          <t>08-09-2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2026/09/Ingot-01-09-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-8-9-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
@@ -731,22 +731,22 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>360.15</v>
+        <v>361.65</v>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>28-08-2026</t>
+          <t>02-09-2026</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-08-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/09/Ingot-01-09-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
@@ -759,22 +759,22 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>356.25</v>
+        <v>360.15</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>21-08-2026</t>
+          <t>28-08-2026</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-21-08-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-08-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
@@ -787,22 +787,22 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>362.35</v>
+        <v>356.25</v>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>15-08-2026</t>
+          <t>21-08-2026</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-15-08-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-21-08-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
@@ -815,22 +815,22 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>375.25</v>
+        <v>362.35</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>12-08-2026</t>
+          <t>15-08-2026</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-12-08-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-15-08-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
@@ -843,22 +843,22 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>363.35</v>
+        <v>375.25</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>01-08-2026</t>
+          <t>12-08-2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-08-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-12-08-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
@@ -871,22 +871,22 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>354.95</v>
+        <v>363.35</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>29-07-2026</t>
+          <t>01-08-2026</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-08-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
@@ -899,22 +899,22 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>361.15</v>
+        <v>354.95</v>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>24-07-2026</t>
+          <t>29-07-2026</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-07-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
@@ -927,22 +927,22 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>356.35</v>
+        <v>361.15</v>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>18-07-2026</t>
+          <t>24-07-2026</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-07-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
@@ -955,22 +955,22 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>352.85</v>
+        <v>356.35</v>
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>11-07-2026</t>
+          <t>18-07-2026</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
@@ -983,22 +983,22 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>349.05</v>
+        <v>352.85</v>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>08-07-2026</t>
+          <t>11-07-2026</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-08-07-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
@@ -1011,22 +1011,22 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>344.05</v>
+        <v>349.05</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>01-07-2026</t>
+          <t>08-07-2026</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-08-07-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
@@ -1039,22 +1039,22 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>349.05</v>
+        <v>344.05</v>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>29-06-2026</t>
+          <t>01-07-2026</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
@@ -1071,18 +1071,18 @@
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>26-06-2026</t>
+          <t>29-06-2026</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
@@ -1095,22 +1095,22 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>376.55</v>
+        <v>349.05</v>
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>18-06-2026</t>
+          <t>26-06-2026</t>
         </is>
       </c>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
@@ -1138,7 +1138,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
@@ -1151,22 +1151,22 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>393.85</v>
+        <v>376.55</v>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>13-06-2026</t>
+          <t>18-06-2026</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
@@ -1179,22 +1179,22 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>402.35</v>
+        <v>393.85</v>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>10-06-2026</t>
+          <t>13-06-2026</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-10-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
@@ -1207,22 +1207,22 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>416.35</v>
+        <v>402.35</v>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>05-06-2026</t>
+          <t>10-06-2026</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-10-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
@@ -1235,22 +1235,22 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>412.55</v>
+        <v>416.35</v>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>01-06-2026</t>
+          <t>05-06-2026</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
@@ -1263,22 +1263,22 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>411.05</v>
+        <v>412.55</v>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>27-05-2026</t>
+          <t>01-06-2026</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
@@ -1291,22 +1291,22 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>404.95</v>
+        <v>411.05</v>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>20-05-2026</t>
+          <t>27-05-2026</t>
         </is>
       </c>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
@@ -1319,22 +1319,22 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>408.85</v>
+        <v>404.95</v>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>14-05-2026</t>
+          <t>20-05-2026</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
@@ -1347,22 +1347,22 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>390.05</v>
+        <v>408.85</v>
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>01-05-2026</t>
+          <t>14-05-2026</t>
         </is>
       </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
@@ -1375,22 +1375,22 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>392.55</v>
+        <v>390.05</v>
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>24-04-2026</t>
+          <t>01-05-2026</t>
         </is>
       </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
@@ -1403,22 +1403,22 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>383.65</v>
+        <v>392.55</v>
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>16-04-2026</t>
+          <t>24-04-2026</t>
         </is>
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
@@ -1431,22 +1431,22 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>373.55</v>
+        <v>383.65</v>
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>03-04-2026</t>
+          <t>16-04-2026</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
@@ -1459,22 +1459,22 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>357.05</v>
+        <v>373.55</v>
       </c>
       <c r="E37" s="1" t="inlineStr">
         <is>
-          <t>28-03-2026</t>
+          <t>03-04-2026</t>
         </is>
       </c>
       <c r="F37" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
@@ -1487,22 +1487,22 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>350.45</v>
+        <v>357.05</v>
       </c>
       <c r="E38" s="1" t="inlineStr">
         <is>
-          <t>24-03-2026</t>
+          <t>28-03-2026</t>
         </is>
       </c>
       <c r="F38" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
@@ -1515,22 +1515,22 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>360.05</v>
+        <v>350.45</v>
       </c>
       <c r="E39" s="1" t="inlineStr">
         <is>
-          <t>19-03-2026</t>
+          <t>24-03-2026</t>
         </is>
       </c>
       <c r="F39" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B40" s="1" t="inlineStr">
         <is>
@@ -1543,22 +1543,22 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>372.05</v>
+        <v>360.05</v>
       </c>
       <c r="E40" s="1" t="inlineStr">
         <is>
-          <t>14-03-2026</t>
+          <t>19-03-2026</t>
         </is>
       </c>
       <c r="F40" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B41" s="1" t="inlineStr">
         <is>
@@ -1571,22 +1571,22 @@
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>358.75</v>
+        <v>372.05</v>
       </c>
       <c r="E41" s="1" t="inlineStr">
         <is>
-          <t>11-03-2026</t>
+          <t>14-03-2026</t>
         </is>
       </c>
       <c r="F41" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B42" s="1" t="inlineStr">
         <is>
@@ -1599,22 +1599,22 @@
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>347.25</v>
+        <v>358.75</v>
       </c>
       <c r="E42" s="1" t="inlineStr">
         <is>
-          <t>06-03-2026</t>
+          <t>11-03-2026</t>
         </is>
       </c>
       <c r="F42" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B43" s="1" t="inlineStr">
         <is>
@@ -1627,22 +1627,22 @@
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>339.45</v>
+        <v>347.25</v>
       </c>
       <c r="E43" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>06-03-2026</t>
         </is>
       </c>
       <c r="F43" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B44" s="1" t="inlineStr">
         <is>
@@ -1655,22 +1655,22 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>330.95</v>
+        <v>339.45</v>
       </c>
       <c r="E44" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F44" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B45" s="1" t="inlineStr">
         <is>
@@ -1683,22 +1683,22 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>323.05</v>
+        <v>330.95</v>
       </c>
       <c r="E45" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="F45" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B46" s="1" t="inlineStr">
         <is>
@@ -1711,22 +1711,22 @@
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>316.15</v>
+        <v>323.05</v>
       </c>
       <c r="E46" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="F46" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B47" s="1" t="inlineStr">
         <is>
@@ -1739,22 +1739,22 @@
         </is>
       </c>
       <c r="D47" s="2" t="n">
-        <v>323.75</v>
+        <v>316.15</v>
       </c>
       <c r="E47" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="F47" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B48" s="1" t="inlineStr">
         <is>
@@ -1767,22 +1767,22 @@
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>318.05</v>
+        <v>323.75</v>
       </c>
       <c r="E48" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="F48" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B49" s="1" t="inlineStr">
         <is>
@@ -1795,22 +1795,22 @@
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>320.45</v>
+        <v>318.05</v>
       </c>
       <c r="E49" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="F49" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B50" s="1" t="inlineStr">
         <is>
@@ -1823,22 +1823,22 @@
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E50" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F50" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B51" s="1" t="inlineStr">
         <is>
@@ -1851,22 +1851,22 @@
         </is>
       </c>
       <c r="D51" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E51" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F51" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="B52" s="1" t="inlineStr">
         <is>
@@ -1879,22 +1879,22 @@
         </is>
       </c>
       <c r="D52" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E52" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F52" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B53" s="1" t="inlineStr">
         <is>
@@ -1907,22 +1907,22 @@
         </is>
       </c>
       <c r="D53" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E53" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F53" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B54" s="1" t="inlineStr">
         <is>
@@ -1935,22 +1935,22 @@
         </is>
       </c>
       <c r="D54" s="2" t="n">
-        <v>307.25</v>
+        <v>320.05</v>
       </c>
       <c r="E54" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="F54" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B55" s="1" t="inlineStr">
         <is>
@@ -1963,22 +1963,22 @@
         </is>
       </c>
       <c r="D55" s="2" t="n">
-        <v>301.65</v>
+        <v>307.25</v>
       </c>
       <c r="E55" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F55" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B56" s="1" t="inlineStr">
         <is>
@@ -1991,22 +1991,22 @@
         </is>
       </c>
       <c r="D56" s="2" t="n">
-        <v>296.05</v>
+        <v>301.65</v>
       </c>
       <c r="E56" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="F56" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B57" s="1" t="inlineStr">
         <is>
@@ -2019,22 +2019,22 @@
         </is>
       </c>
       <c r="D57" s="2" t="n">
-        <v>290.95</v>
+        <v>296.05</v>
       </c>
       <c r="E57" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="F57" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B58" s="1" t="inlineStr">
         <is>
@@ -2047,22 +2047,22 @@
         </is>
       </c>
       <c r="D58" s="2" t="n">
-        <v>283.55</v>
+        <v>290.95</v>
       </c>
       <c r="E58" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="F58" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B59" s="1" t="inlineStr">
         <is>
@@ -2075,22 +2075,22 @@
         </is>
       </c>
       <c r="D59" s="2" t="n">
-        <v>281.95</v>
+        <v>283.55</v>
       </c>
       <c r="E59" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="F59" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B60" s="1" t="inlineStr">
         <is>
@@ -2103,22 +2103,22 @@
         </is>
       </c>
       <c r="D60" s="2" t="n">
-        <v>292.65</v>
+        <v>281.95</v>
       </c>
       <c r="E60" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="F60" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B61" s="1" t="inlineStr">
         <is>
@@ -2131,22 +2131,22 @@
         </is>
       </c>
       <c r="D61" s="2" t="n">
-        <v>296.05</v>
+        <v>292.65</v>
       </c>
       <c r="E61" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="F61" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B62" s="1" t="inlineStr">
         <is>
@@ -2159,22 +2159,22 @@
         </is>
       </c>
       <c r="D62" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E62" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F62" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="1" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B63" s="1" t="inlineStr">
         <is>
@@ -2187,22 +2187,22 @@
         </is>
       </c>
       <c r="D63" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E63" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F63" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="1" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B64" s="1" t="inlineStr">
         <is>
@@ -2215,22 +2215,22 @@
         </is>
       </c>
       <c r="D64" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E64" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F64" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="1" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B65" s="1" t="inlineStr">
         <is>
@@ -2243,22 +2243,22 @@
         </is>
       </c>
       <c r="D65" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E65" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F65" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="1" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B66" s="1" t="inlineStr">
         <is>
@@ -2271,22 +2271,22 @@
         </is>
       </c>
       <c r="D66" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E66" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F66" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="1" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B67" s="1" t="inlineStr">
         <is>
@@ -2299,22 +2299,22 @@
         </is>
       </c>
       <c r="D67" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E67" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F67" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="1" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B68" s="1" t="inlineStr">
         <is>
@@ -2327,22 +2327,22 @@
         </is>
       </c>
       <c r="D68" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E68" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F68" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="1" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B69" s="1" t="inlineStr">
         <is>
@@ -2355,22 +2355,22 @@
         </is>
       </c>
       <c r="D69" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E69" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F69" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="1" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B70" s="1" t="inlineStr">
         <is>
@@ -2383,22 +2383,22 @@
         </is>
       </c>
       <c r="D70" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E70" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F70" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="1" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B71" s="1" t="inlineStr">
         <is>
@@ -2411,22 +2411,22 @@
         </is>
       </c>
       <c r="D71" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E71" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F71" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="1" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B72" s="1" t="inlineStr">
         <is>
@@ -2439,22 +2439,22 @@
         </is>
       </c>
       <c r="D72" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E72" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F72" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B73" s="1" t="inlineStr">
         <is>
@@ -2467,22 +2467,22 @@
         </is>
       </c>
       <c r="D73" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E73" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F73" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B74" s="1" t="inlineStr">
         <is>
@@ -2495,22 +2495,22 @@
         </is>
       </c>
       <c r="D74" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E74" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F74" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="1" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B75" s="1" t="inlineStr">
         <is>
@@ -2523,22 +2523,22 @@
         </is>
       </c>
       <c r="D75" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E75" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F75" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B76" s="1" t="inlineStr">
         <is>
@@ -2551,42 +2551,70 @@
         </is>
       </c>
       <c r="D76" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E76" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F76" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B77" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C77" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="n">
+        <v>269.45</v>
+      </c>
+      <c r="E77" s="1" t="inlineStr">
+        <is>
+          <t>15-08-2025</t>
+        </is>
+      </c>
+      <c r="F77" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B77" s="1" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C77" s="1" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D77" s="2" t="n">
+      <c r="B78" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C78" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="n">
         <v>268.25</v>
       </c>
-      <c r="E77" s="1" t="inlineStr">
+      <c r="E78" s="1" t="inlineStr">
         <is>
           <t>07-08-2025</t>
         </is>
       </c>
-      <c r="F77" s="1" t="inlineStr">
+      <c r="F78" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
@@ -2670,6 +2698,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F75" r:id="rId74"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F76" r:id="rId75"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F77" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F78" r:id="rId77"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-29 10:16:11 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F78"/>
+  <dimension ref="A1:F79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -466,7 +466,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -479,22 +479,22 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>339.85</v>
+        <v>346.75</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>24-10-2026</t>
+          <t>29-10-2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-10-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-10-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
@@ -507,22 +507,22 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>335.75</v>
+        <v>339.85</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>16-10-2026</t>
+          <t>24-10-2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-10-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-10-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
@@ -535,22 +535,22 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>343.65</v>
+        <v>335.75</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>13-10-2026</t>
+          <t>16-10-2026</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-10-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-10-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
@@ -563,22 +563,22 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>351.25</v>
+        <v>343.65</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>01-10-2026</t>
+          <t>13-10-2026</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-10-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
@@ -591,22 +591,22 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>362.75</v>
+        <v>351.25</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>24-09-2026</t>
+          <t>01-10-2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-09-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
@@ -619,22 +619,22 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>367.65</v>
+        <v>362.75</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>19-09-2026</t>
+          <t>24-09-2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-09-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-09-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
@@ -647,22 +647,22 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>365.55</v>
+        <v>367.65</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>16-09-2026</t>
+          <t>19-09-2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-09-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-09-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
@@ -675,22 +675,22 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>371.55</v>
+        <v>365.55</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>11-09-2026</t>
+          <t>16-09-2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-09-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-09-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
@@ -703,22 +703,22 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>365.25</v>
+        <v>371.55</v>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>08-09-2026</t>
+          <t>11-09-2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-8-9-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-09-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
@@ -731,22 +731,22 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>361.65</v>
+        <v>365.25</v>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>02-09-2026</t>
+          <t>08-09-2026</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2026/09/Ingot-01-09-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-8-9-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
@@ -759,22 +759,22 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>360.15</v>
+        <v>361.65</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>28-08-2026</t>
+          <t>02-09-2026</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-08-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/09/Ingot-01-09-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
@@ -787,22 +787,22 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>356.25</v>
+        <v>360.15</v>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>21-08-2026</t>
+          <t>28-08-2026</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-21-08-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-08-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
@@ -815,22 +815,22 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>362.35</v>
+        <v>356.25</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>15-08-2026</t>
+          <t>21-08-2026</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-15-08-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-21-08-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
@@ -843,22 +843,22 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>375.25</v>
+        <v>362.35</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>12-08-2026</t>
+          <t>15-08-2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-12-08-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-15-08-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
@@ -871,22 +871,22 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>363.35</v>
+        <v>375.25</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>01-08-2026</t>
+          <t>12-08-2026</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-08-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-12-08-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
@@ -899,22 +899,22 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>354.95</v>
+        <v>363.35</v>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>29-07-2026</t>
+          <t>01-08-2026</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-08-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
@@ -927,22 +927,22 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>361.15</v>
+        <v>354.95</v>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>24-07-2026</t>
+          <t>29-07-2026</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-07-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
@@ -955,22 +955,22 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>356.35</v>
+        <v>361.15</v>
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>18-07-2026</t>
+          <t>24-07-2026</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-07-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
@@ -983,22 +983,22 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>352.85</v>
+        <v>356.35</v>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>11-07-2026</t>
+          <t>18-07-2026</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
@@ -1011,22 +1011,22 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>349.05</v>
+        <v>352.85</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>08-07-2026</t>
+          <t>11-07-2026</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-08-07-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
@@ -1039,22 +1039,22 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>344.05</v>
+        <v>349.05</v>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>01-07-2026</t>
+          <t>08-07-2026</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-08-07-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
@@ -1067,22 +1067,22 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>349.05</v>
+        <v>344.05</v>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>29-06-2026</t>
+          <t>01-07-2026</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
@@ -1099,18 +1099,18 @@
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>26-06-2026</t>
+          <t>29-06-2026</t>
         </is>
       </c>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
@@ -1123,22 +1123,22 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>376.55</v>
+        <v>349.05</v>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>18-06-2026</t>
+          <t>26-06-2026</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
@@ -1166,7 +1166,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
@@ -1179,22 +1179,22 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>393.85</v>
+        <v>376.55</v>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>13-06-2026</t>
+          <t>18-06-2026</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
@@ -1207,22 +1207,22 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>402.35</v>
+        <v>393.85</v>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>10-06-2026</t>
+          <t>13-06-2026</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-10-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
@@ -1235,22 +1235,22 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>416.35</v>
+        <v>402.35</v>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>05-06-2026</t>
+          <t>10-06-2026</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-10-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
@@ -1263,22 +1263,22 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>412.55</v>
+        <v>416.35</v>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>01-06-2026</t>
+          <t>05-06-2026</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
@@ -1291,22 +1291,22 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>411.05</v>
+        <v>412.55</v>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>27-05-2026</t>
+          <t>01-06-2026</t>
         </is>
       </c>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
@@ -1319,22 +1319,22 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>404.95</v>
+        <v>411.05</v>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>20-05-2026</t>
+          <t>27-05-2026</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
@@ -1347,22 +1347,22 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>408.85</v>
+        <v>404.95</v>
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>14-05-2026</t>
+          <t>20-05-2026</t>
         </is>
       </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
@@ -1375,22 +1375,22 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>390.05</v>
+        <v>408.85</v>
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>01-05-2026</t>
+          <t>14-05-2026</t>
         </is>
       </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
@@ -1403,22 +1403,22 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>392.55</v>
+        <v>390.05</v>
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>24-04-2026</t>
+          <t>01-05-2026</t>
         </is>
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
@@ -1431,22 +1431,22 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>383.65</v>
+        <v>392.55</v>
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>16-04-2026</t>
+          <t>24-04-2026</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
@@ -1459,22 +1459,22 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>373.55</v>
+        <v>383.65</v>
       </c>
       <c r="E37" s="1" t="inlineStr">
         <is>
-          <t>03-04-2026</t>
+          <t>16-04-2026</t>
         </is>
       </c>
       <c r="F37" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
@@ -1487,22 +1487,22 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>357.05</v>
+        <v>373.55</v>
       </c>
       <c r="E38" s="1" t="inlineStr">
         <is>
-          <t>28-03-2026</t>
+          <t>03-04-2026</t>
         </is>
       </c>
       <c r="F38" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
@@ -1515,22 +1515,22 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>350.45</v>
+        <v>357.05</v>
       </c>
       <c r="E39" s="1" t="inlineStr">
         <is>
-          <t>24-03-2026</t>
+          <t>28-03-2026</t>
         </is>
       </c>
       <c r="F39" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B40" s="1" t="inlineStr">
         <is>
@@ -1543,22 +1543,22 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>360.05</v>
+        <v>350.45</v>
       </c>
       <c r="E40" s="1" t="inlineStr">
         <is>
-          <t>19-03-2026</t>
+          <t>24-03-2026</t>
         </is>
       </c>
       <c r="F40" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B41" s="1" t="inlineStr">
         <is>
@@ -1571,22 +1571,22 @@
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>372.05</v>
+        <v>360.05</v>
       </c>
       <c r="E41" s="1" t="inlineStr">
         <is>
-          <t>14-03-2026</t>
+          <t>19-03-2026</t>
         </is>
       </c>
       <c r="F41" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B42" s="1" t="inlineStr">
         <is>
@@ -1599,22 +1599,22 @@
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>358.75</v>
+        <v>372.05</v>
       </c>
       <c r="E42" s="1" t="inlineStr">
         <is>
-          <t>11-03-2026</t>
+          <t>14-03-2026</t>
         </is>
       </c>
       <c r="F42" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B43" s="1" t="inlineStr">
         <is>
@@ -1627,22 +1627,22 @@
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>347.25</v>
+        <v>358.75</v>
       </c>
       <c r="E43" s="1" t="inlineStr">
         <is>
-          <t>06-03-2026</t>
+          <t>11-03-2026</t>
         </is>
       </c>
       <c r="F43" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B44" s="1" t="inlineStr">
         <is>
@@ -1655,22 +1655,22 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>339.45</v>
+        <v>347.25</v>
       </c>
       <c r="E44" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>06-03-2026</t>
         </is>
       </c>
       <c r="F44" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B45" s="1" t="inlineStr">
         <is>
@@ -1683,22 +1683,22 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>330.95</v>
+        <v>339.45</v>
       </c>
       <c r="E45" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F45" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B46" s="1" t="inlineStr">
         <is>
@@ -1711,22 +1711,22 @@
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>323.05</v>
+        <v>330.95</v>
       </c>
       <c r="E46" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="F46" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B47" s="1" t="inlineStr">
         <is>
@@ -1739,22 +1739,22 @@
         </is>
       </c>
       <c r="D47" s="2" t="n">
-        <v>316.15</v>
+        <v>323.05</v>
       </c>
       <c r="E47" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="F47" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B48" s="1" t="inlineStr">
         <is>
@@ -1767,22 +1767,22 @@
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>323.75</v>
+        <v>316.15</v>
       </c>
       <c r="E48" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="F48" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B49" s="1" t="inlineStr">
         <is>
@@ -1795,22 +1795,22 @@
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>318.05</v>
+        <v>323.75</v>
       </c>
       <c r="E49" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="F49" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B50" s="1" t="inlineStr">
         <is>
@@ -1823,22 +1823,22 @@
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>320.45</v>
+        <v>318.05</v>
       </c>
       <c r="E50" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="F50" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B51" s="1" t="inlineStr">
         <is>
@@ -1851,22 +1851,22 @@
         </is>
       </c>
       <c r="D51" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E51" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F51" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B52" s="1" t="inlineStr">
         <is>
@@ -1879,22 +1879,22 @@
         </is>
       </c>
       <c r="D52" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E52" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F52" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="B53" s="1" t="inlineStr">
         <is>
@@ -1907,22 +1907,22 @@
         </is>
       </c>
       <c r="D53" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E53" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F53" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B54" s="1" t="inlineStr">
         <is>
@@ -1935,22 +1935,22 @@
         </is>
       </c>
       <c r="D54" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E54" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F54" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B55" s="1" t="inlineStr">
         <is>
@@ -1963,22 +1963,22 @@
         </is>
       </c>
       <c r="D55" s="2" t="n">
-        <v>307.25</v>
+        <v>320.05</v>
       </c>
       <c r="E55" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="F55" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B56" s="1" t="inlineStr">
         <is>
@@ -1991,22 +1991,22 @@
         </is>
       </c>
       <c r="D56" s="2" t="n">
-        <v>301.65</v>
+        <v>307.25</v>
       </c>
       <c r="E56" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F56" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B57" s="1" t="inlineStr">
         <is>
@@ -2019,22 +2019,22 @@
         </is>
       </c>
       <c r="D57" s="2" t="n">
-        <v>296.05</v>
+        <v>301.65</v>
       </c>
       <c r="E57" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="F57" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B58" s="1" t="inlineStr">
         <is>
@@ -2047,22 +2047,22 @@
         </is>
       </c>
       <c r="D58" s="2" t="n">
-        <v>290.95</v>
+        <v>296.05</v>
       </c>
       <c r="E58" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="F58" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B59" s="1" t="inlineStr">
         <is>
@@ -2075,22 +2075,22 @@
         </is>
       </c>
       <c r="D59" s="2" t="n">
-        <v>283.55</v>
+        <v>290.95</v>
       </c>
       <c r="E59" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="F59" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B60" s="1" t="inlineStr">
         <is>
@@ -2103,22 +2103,22 @@
         </is>
       </c>
       <c r="D60" s="2" t="n">
-        <v>281.95</v>
+        <v>283.55</v>
       </c>
       <c r="E60" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="F60" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B61" s="1" t="inlineStr">
         <is>
@@ -2131,22 +2131,22 @@
         </is>
       </c>
       <c r="D61" s="2" t="n">
-        <v>292.65</v>
+        <v>281.95</v>
       </c>
       <c r="E61" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="F61" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B62" s="1" t="inlineStr">
         <is>
@@ -2159,22 +2159,22 @@
         </is>
       </c>
       <c r="D62" s="2" t="n">
-        <v>296.05</v>
+        <v>292.65</v>
       </c>
       <c r="E62" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="F62" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="1" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B63" s="1" t="inlineStr">
         <is>
@@ -2187,22 +2187,22 @@
         </is>
       </c>
       <c r="D63" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E63" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F63" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="1" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B64" s="1" t="inlineStr">
         <is>
@@ -2215,22 +2215,22 @@
         </is>
       </c>
       <c r="D64" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E64" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F64" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="1" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B65" s="1" t="inlineStr">
         <is>
@@ -2243,22 +2243,22 @@
         </is>
       </c>
       <c r="D65" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E65" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F65" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="1" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B66" s="1" t="inlineStr">
         <is>
@@ -2271,22 +2271,22 @@
         </is>
       </c>
       <c r="D66" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E66" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F66" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="1" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B67" s="1" t="inlineStr">
         <is>
@@ -2299,22 +2299,22 @@
         </is>
       </c>
       <c r="D67" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E67" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F67" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="1" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B68" s="1" t="inlineStr">
         <is>
@@ -2327,22 +2327,22 @@
         </is>
       </c>
       <c r="D68" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E68" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F68" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="1" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B69" s="1" t="inlineStr">
         <is>
@@ -2355,22 +2355,22 @@
         </is>
       </c>
       <c r="D69" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E69" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F69" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="1" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B70" s="1" t="inlineStr">
         <is>
@@ -2383,22 +2383,22 @@
         </is>
       </c>
       <c r="D70" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E70" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F70" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="1" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B71" s="1" t="inlineStr">
         <is>
@@ -2411,22 +2411,22 @@
         </is>
       </c>
       <c r="D71" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E71" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F71" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="1" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B72" s="1" t="inlineStr">
         <is>
@@ -2439,22 +2439,22 @@
         </is>
       </c>
       <c r="D72" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E72" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F72" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="1" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B73" s="1" t="inlineStr">
         <is>
@@ -2467,22 +2467,22 @@
         </is>
       </c>
       <c r="D73" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E73" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F73" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B74" s="1" t="inlineStr">
         <is>
@@ -2495,22 +2495,22 @@
         </is>
       </c>
       <c r="D74" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E74" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F74" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B75" s="1" t="inlineStr">
         <is>
@@ -2523,22 +2523,22 @@
         </is>
       </c>
       <c r="D75" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E75" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F75" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="1" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B76" s="1" t="inlineStr">
         <is>
@@ -2551,22 +2551,22 @@
         </is>
       </c>
       <c r="D76" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E76" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F76" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B77" s="1" t="inlineStr">
         <is>
@@ -2579,42 +2579,70 @@
         </is>
       </c>
       <c r="D77" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E77" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F77" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B78" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C78" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="n">
+        <v>269.45</v>
+      </c>
+      <c r="E78" s="1" t="inlineStr">
+        <is>
+          <t>15-08-2025</t>
+        </is>
+      </c>
+      <c r="F78" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B78" s="1" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C78" s="1" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D78" s="2" t="n">
+      <c r="B79" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C79" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="n">
         <v>268.25</v>
       </c>
-      <c r="E78" s="1" t="inlineStr">
+      <c r="E79" s="1" t="inlineStr">
         <is>
           <t>07-08-2025</t>
         </is>
       </c>
-      <c r="F78" s="1" t="inlineStr">
+      <c r="F79" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
@@ -2699,6 +2727,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F76" r:id="rId75"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F77" r:id="rId76"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F78" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F79" r:id="rId78"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>